<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:15:20 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -949,10 +949,10 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1642,10 +1642,10 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1993,10 +1993,10 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2458,10 +2458,10 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3037,10 +3037,10 @@
         <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4500,7 +4500,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4642,10 +4642,10 @@
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5221,10 +5221,10 @@
         <v>1</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6684,7 +6684,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6912,7 +6912,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7026,7 +7026,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7368,7 +7368,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7482,7 +7482,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7624,10 +7624,10 @@
         <v>0</v>
       </c>
       <c r="I62" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
@@ -7719,7 +7719,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7833,7 +7833,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7947,7 +7947,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7975,10 +7975,10 @@
         <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -8070,7 +8070,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8184,7 +8184,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8298,7 +8298,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8412,7 +8412,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8440,10 +8440,10 @@
         <v>1</v>
       </c>
       <c r="I69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -8535,7 +8535,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8649,7 +8649,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8763,7 +8763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8877,7 +8877,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8905,10 +8905,10 @@
         <v>0</v>
       </c>
       <c r="I73" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -9000,7 +9000,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9028,10 +9028,10 @@
         <v>1</v>
       </c>
       <c r="I74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -9123,7 +9123,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9237,7 +9237,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9465,7 +9465,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9579,7 +9579,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9693,7 +9693,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9807,7 +9807,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9921,7 +9921,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10035,7 +10035,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10149,7 +10149,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10263,7 +10263,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10377,7 +10377,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10491,7 +10491,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10605,7 +10605,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10633,10 +10633,10 @@
         <v>0</v>
       </c>
       <c r="I88" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -10728,7 +10728,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10842,7 +10842,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11070,7 +11070,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11184,7 +11184,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11298,7 +11298,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11412,7 +11412,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11554,10 +11554,10 @@
         <v>1</v>
       </c>
       <c r="I96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12133,10 +12133,10 @@
         <v>0</v>
       </c>
       <c r="I101" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
@@ -12228,7 +12228,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12342,7 +12342,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12570,7 +12570,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12684,7 +12684,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12798,7 +12798,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12912,7 +12912,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12940,10 +12940,10 @@
         <v>1</v>
       </c>
       <c r="I108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -13035,7 +13035,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13149,7 +13149,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13263,7 +13263,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13491,7 +13491,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13605,7 +13605,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13633,10 +13633,10 @@
         <v>0</v>
       </c>
       <c r="I114" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -13728,7 +13728,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13842,7 +13842,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13870,10 +13870,10 @@
         <v>1</v>
       </c>
       <c r="I116" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J116" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -13965,7 +13965,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14193,7 +14193,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14307,7 +14307,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14535,7 +14535,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14649,7 +14649,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14763,7 +14763,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14877,7 +14877,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15105,7 +15105,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15219,7 +15219,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15247,10 +15247,10 @@
         <v>1</v>
       </c>
       <c r="I128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15342,7 +15342,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15456,7 +15456,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15570,7 +15570,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15684,7 +15684,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15912,7 +15912,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16026,7 +16026,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16140,7 +16140,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16368,7 +16368,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16482,7 +16482,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16596,7 +16596,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16824,7 +16824,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16938,7 +16938,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17052,7 +17052,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17166,7 +17166,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17280,7 +17280,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17308,10 +17308,10 @@
         <v>1</v>
       </c>
       <c r="I146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K146" t="inlineStr">
         <is>
@@ -17403,7 +17403,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17517,7 +17517,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17745,7 +17745,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17973,7 +17973,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18087,7 +18087,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18315,7 +18315,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18429,7 +18429,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18457,10 +18457,10 @@
         <v>0</v>
       </c>
       <c r="I156" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J156" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -18552,7 +18552,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18580,10 +18580,10 @@
         <v>0</v>
       </c>
       <c r="I157" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -18675,7 +18675,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18703,10 +18703,10 @@
         <v>0</v>
       </c>
       <c r="I158" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J158" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18826,10 +18826,10 @@
         <v>0</v>
       </c>
       <c r="I159" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19263,7 +19263,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19377,7 +19377,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19605,7 +19605,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20175,7 +20175,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20203,10 +20203,10 @@
         <v>1</v>
       </c>
       <c r="I171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20298,7 +20298,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20326,10 +20326,10 @@
         <v>1</v>
       </c>
       <c r="I172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20421,7 +20421,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20763,7 +20763,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20877,7 +20877,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20991,7 +20991,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21105,7 +21105,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21333,7 +21333,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21561,7 +21561,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21789,7 +21789,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21903,7 +21903,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22017,7 +22017,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22131,7 +22131,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22245,7 +22245,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22473,7 +22473,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22587,7 +22587,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22615,10 +22615,10 @@
         <v>1</v>
       </c>
       <c r="I192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K192" t="inlineStr">
         <is>
@@ -22710,7 +22710,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22824,7 +22824,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22938,7 +22938,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23052,7 +23052,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23166,7 +23166,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23280,7 +23280,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23394,7 +23394,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23508,7 +23508,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23622,7 +23622,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23736,7 +23736,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23850,7 +23850,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23964,7 +23964,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24078,7 +24078,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24192,7 +24192,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24306,7 +24306,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24420,7 +24420,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24534,7 +24534,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24648,7 +24648,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24762,7 +24762,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24876,7 +24876,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24990,7 +24990,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25104,7 +25104,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25218,7 +25218,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25332,7 +25332,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25446,7 +25446,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25560,7 +25560,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25674,7 +25674,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25788,7 +25788,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25902,7 +25902,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26016,7 +26016,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26130,7 +26130,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26244,7 +26244,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26358,7 +26358,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26472,7 +26472,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26586,7 +26586,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26700,7 +26700,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26728,10 +26728,10 @@
         <v>0</v>
       </c>
       <c r="I228" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J228" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K228" t="inlineStr">
         <is>
@@ -26823,7 +26823,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26937,7 +26937,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27051,7 +27051,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27165,7 +27165,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27279,7 +27279,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27307,10 +27307,10 @@
         <v>1</v>
       </c>
       <c r="I233" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J233" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K233" t="inlineStr">
         <is>
@@ -27402,7 +27402,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27430,10 +27430,10 @@
         <v>1</v>
       </c>
       <c r="I234" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J234" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K234" t="inlineStr">
         <is>
@@ -27525,7 +27525,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27553,10 +27553,10 @@
         <v>1</v>
       </c>
       <c r="I235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K235" t="inlineStr">
         <is>
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27762,7 +27762,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27876,7 +27876,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27990,7 +27990,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28104,7 +28104,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28218,7 +28218,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28332,7 +28332,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28446,7 +28446,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28560,7 +28560,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28674,7 +28674,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28788,7 +28788,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28902,7 +28902,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29016,7 +29016,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29130,7 +29130,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29244,7 +29244,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29472,7 +29472,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29586,7 +29586,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29700,7 +29700,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29814,7 +29814,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29928,7 +29928,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30042,7 +30042,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30156,7 +30156,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30270,7 +30270,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30384,7 +30384,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30498,7 +30498,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30612,7 +30612,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30726,7 +30726,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30840,7 +30840,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30954,7 +30954,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31068,7 +31068,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31182,7 +31182,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31296,7 +31296,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31410,7 +31410,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31524,7 +31524,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31638,7 +31638,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31752,7 +31752,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31866,7 +31866,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31980,7 +31980,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32094,7 +32094,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32208,7 +32208,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32322,7 +32322,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32436,7 +32436,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32464,10 +32464,10 @@
         <v>1</v>
       </c>
       <c r="I278" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J278" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K278" t="inlineStr">
         <is>
@@ -32559,7 +32559,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32587,10 +32587,10 @@
         <v>1</v>
       </c>
       <c r="I279" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J279" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K279" t="inlineStr">
         <is>
@@ -32682,7 +32682,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32710,10 +32710,10 @@
         <v>1</v>
       </c>
       <c r="I280" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J280" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K280" t="inlineStr">
         <is>
@@ -32805,7 +32805,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32833,10 +32833,10 @@
         <v>1</v>
       </c>
       <c r="I281" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J281" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K281" t="inlineStr">
         <is>
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33042,7 +33042,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33156,7 +33156,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33270,7 +33270,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33384,7 +33384,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33498,7 +33498,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33612,7 +33612,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33726,7 +33726,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33840,7 +33840,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33954,7 +33954,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34068,7 +34068,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34182,7 +34182,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34296,7 +34296,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34410,7 +34410,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34524,7 +34524,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34638,7 +34638,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34752,7 +34752,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34866,7 +34866,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34980,7 +34980,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35094,7 +35094,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35208,7 +35208,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35322,7 +35322,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35436,7 +35436,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:16 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35550,7 +35550,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:16 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35664,7 +35664,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35692,10 +35692,10 @@
         <v>0</v>
       </c>
       <c r="I306" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J306" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K306" t="inlineStr">
         <is>
@@ -35787,7 +35787,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35901,7 +35901,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36015,7 +36015,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36129,7 +36129,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36243,7 +36243,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36357,7 +36357,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36471,7 +36471,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36585,7 +36585,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36699,7 +36699,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36813,7 +36813,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36927,7 +36927,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37041,7 +37041,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37155,7 +37155,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37269,7 +37269,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37383,7 +37383,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37497,7 +37497,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37611,7 +37611,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37725,7 +37725,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37839,7 +37839,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37953,7 +37953,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:18 PM PT</t>
+          <t>2026-07-11 08:15:18 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -38067,7 +38067,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:19 PM PT</t>
+          <t>2026-07-11 08:15:19 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38095,10 +38095,10 @@
         <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K327" t="inlineStr">
         <is>
@@ -38190,7 +38190,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38304,7 +38304,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:13:17 PM PT</t>
+          <t>2026-07-11 08:15:17 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:23:19 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Live Fantasy Scores'!$A$1:$AG$329</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Live Fantasy Scores'!$A$1:$AG$330</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,14 +480,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG329"/>
+  <dimension ref="A1:AG330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -934,25 +934,25 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1627,25 +1627,25 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1978,25 +1978,25 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2443,25 +2443,25 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -3034,13 +3034,13 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4500,7 +4500,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4627,25 +4627,25 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -5218,13 +5218,13 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I41" t="n">
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -5260,10 +5260,10 @@
         </is>
       </c>
       <c r="R41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T41" t="n">
         <v>2</v>
@@ -5296,7 +5296,7 @@
         <v>0</v>
       </c>
       <c r="AD41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE41" s="4" t="n">
         <v>14</v>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6355,7 +6355,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -6367,13 +6367,13 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6579,7 +6579,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6807,7 +6807,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7035,7 +7035,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7377,7 +7377,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7605,7 +7605,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7719,7 +7719,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7732,25 +7732,25 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H63" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I63" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -7842,7 +7842,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -7867,13 +7867,13 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8193,7 +8193,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8206,25 +8206,25 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H67" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8316,7 +8316,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8430,7 +8430,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -8683,13 +8683,13 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I71" t="n">
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -8781,7 +8781,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -9009,7 +9009,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9123,7 +9123,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9136,25 +9136,25 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F75" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H75" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J75" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9702,7 +9702,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10272,7 +10272,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10386,7 +10386,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10500,7 +10500,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10728,7 +10728,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10741,25 +10741,25 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H89" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I89" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11092,7 +11092,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -11104,13 +11104,13 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I92" t="n">
         <v>0</v>
       </c>
       <c r="J92" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11316,7 +11316,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11430,7 +11430,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11544,7 +11544,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11772,7 +11772,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11785,7 +11785,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -11797,13 +11797,13 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I98" t="n">
         <v>0</v>
       </c>
       <c r="J98" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -11895,7 +11895,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12123,7 +12123,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12351,7 +12351,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12364,25 +12364,25 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F103" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H103" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I103" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J103" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12588,7 +12588,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12702,7 +12702,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12816,7 +12816,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12930,7 +12930,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13044,7 +13044,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13158,7 +13158,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13386,7 +13386,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13614,7 +13614,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13728,7 +13728,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13741,25 +13741,25 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H115" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I115" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J115" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -13851,7 +13851,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13965,7 +13965,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14193,7 +14193,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14307,7 +14307,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14535,7 +14535,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14649,7 +14649,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14763,7 +14763,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14877,7 +14877,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15105,7 +15105,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15219,7 +15219,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15232,7 +15232,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -15244,13 +15244,13 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I128" t="n">
         <v>0</v>
       </c>
       <c r="J128" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15342,7 +15342,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15456,7 +15456,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15570,7 +15570,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15684,7 +15684,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15912,7 +15912,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16026,7 +16026,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16140,7 +16140,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16368,7 +16368,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16482,7 +16482,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16596,7 +16596,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16824,7 +16824,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16938,7 +16938,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17052,7 +17052,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17166,7 +17166,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17280,7 +17280,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17293,7 +17293,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -17305,13 +17305,13 @@
         </is>
       </c>
       <c r="H146" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I146" t="n">
         <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K146" t="inlineStr">
         <is>
@@ -17403,7 +17403,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17517,7 +17517,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17745,7 +17745,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17973,7 +17973,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18087,7 +18087,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18315,7 +18315,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18429,7 +18429,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18442,25 +18442,25 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F156" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H156" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I156" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J156" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -18552,7 +18552,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18565,25 +18565,25 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F157" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H157" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I157" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J157" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -18675,7 +18675,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18688,25 +18688,25 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F158" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H158" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I158" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J158" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18811,25 +18811,25 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F159" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H159" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I159" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J159" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19263,7 +19263,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19377,7 +19377,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19605,7 +19605,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20175,7 +20175,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20188,7 +20188,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -20200,13 +20200,13 @@
         </is>
       </c>
       <c r="H171" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I171" t="n">
         <v>0</v>
       </c>
       <c r="J171" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20298,7 +20298,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20311,7 +20311,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20323,13 +20323,13 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I172" t="n">
         <v>0</v>
       </c>
       <c r="J172" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20421,7 +20421,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20763,7 +20763,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20877,7 +20877,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20991,7 +20991,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21105,7 +21105,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21333,7 +21333,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21561,7 +21561,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21789,7 +21789,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21903,7 +21903,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22017,7 +22017,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22131,7 +22131,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22245,7 +22245,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22473,7 +22473,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22587,7 +22587,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22600,7 +22600,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -22612,13 +22612,13 @@
         </is>
       </c>
       <c r="H192" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I192" t="n">
         <v>0</v>
       </c>
       <c r="J192" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K192" t="inlineStr">
         <is>
@@ -22710,7 +22710,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22723,7 +22723,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -22735,13 +22735,13 @@
         </is>
       </c>
       <c r="H193" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I193" t="n">
         <v>0</v>
       </c>
       <c r="J193" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K193" t="inlineStr">
         <is>
@@ -22833,7 +22833,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22947,7 +22947,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23061,7 +23061,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23175,7 +23175,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23289,7 +23289,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23403,7 +23403,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23517,7 +23517,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23631,7 +23631,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23745,7 +23745,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23859,7 +23859,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23973,7 +23973,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24087,7 +24087,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24201,7 +24201,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24429,7 +24429,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24543,7 +24543,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24657,7 +24657,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24771,7 +24771,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24885,7 +24885,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24999,7 +24999,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25113,7 +25113,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25227,7 +25227,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25341,7 +25341,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25455,7 +25455,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25569,7 +25569,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25683,7 +25683,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25797,7 +25797,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25911,7 +25911,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26025,7 +26025,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26139,7 +26139,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26253,7 +26253,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26367,7 +26367,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26481,7 +26481,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26595,7 +26595,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26709,7 +26709,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26823,7 +26823,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26836,25 +26836,25 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F229" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H229" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I229" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J229" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K229" t="inlineStr">
         <is>
@@ -26946,7 +26946,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27060,7 +27060,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27174,7 +27174,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27288,7 +27288,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27402,7 +27402,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27415,7 +27415,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F234" t="n">
@@ -27427,13 +27427,13 @@
         </is>
       </c>
       <c r="H234" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I234" t="n">
         <v>0</v>
       </c>
       <c r="J234" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K234" t="inlineStr">
         <is>
@@ -27525,7 +27525,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27538,7 +27538,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F235" t="n">
@@ -27550,13 +27550,13 @@
         </is>
       </c>
       <c r="H235" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I235" t="n">
         <v>0</v>
       </c>
       <c r="J235" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K235" t="inlineStr">
         <is>
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27762,7 +27762,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27876,7 +27876,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27990,7 +27990,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28104,7 +28104,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28218,7 +28218,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28332,7 +28332,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28446,7 +28446,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28560,7 +28560,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28674,7 +28674,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28788,7 +28788,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28902,7 +28902,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29016,7 +29016,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29130,7 +29130,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29244,7 +29244,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29472,7 +29472,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29586,7 +29586,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29700,7 +29700,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29814,7 +29814,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29928,7 +29928,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30042,7 +30042,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30156,7 +30156,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30270,7 +30270,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30384,7 +30384,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30498,7 +30498,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30612,7 +30612,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30726,7 +30726,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30840,7 +30840,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30954,7 +30954,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31068,7 +31068,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31182,7 +31182,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31296,7 +31296,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31410,7 +31410,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31524,7 +31524,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31638,7 +31638,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31752,7 +31752,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31866,7 +31866,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31980,7 +31980,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32094,7 +32094,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32208,7 +32208,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32322,7 +32322,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32436,7 +32436,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32449,7 +32449,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F278" t="n">
@@ -32461,13 +32461,13 @@
         </is>
       </c>
       <c r="H278" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I278" t="n">
         <v>0</v>
       </c>
       <c r="J278" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K278" t="inlineStr">
         <is>
@@ -32559,7 +32559,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32572,7 +32572,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F279" t="n">
@@ -32584,13 +32584,13 @@
         </is>
       </c>
       <c r="H279" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I279" t="n">
         <v>0</v>
       </c>
       <c r="J279" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K279" t="inlineStr">
         <is>
@@ -32682,7 +32682,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32695,7 +32695,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F280" t="n">
@@ -32707,13 +32707,13 @@
         </is>
       </c>
       <c r="H280" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I280" t="n">
         <v>0</v>
       </c>
       <c r="J280" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K280" t="inlineStr">
         <is>
@@ -32805,7 +32805,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32818,7 +32818,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Top 7 | 3 out</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -32830,13 +32830,13 @@
         </is>
       </c>
       <c r="H281" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I281" t="n">
         <v>0</v>
       </c>
       <c r="J281" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K281" t="inlineStr">
         <is>
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33042,7 +33042,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33156,7 +33156,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33270,7 +33270,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33384,7 +33384,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33498,7 +33498,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33612,7 +33612,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33726,7 +33726,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33840,7 +33840,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33954,7 +33954,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34068,7 +34068,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34182,7 +34182,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34296,7 +34296,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34410,7 +34410,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34524,7 +34524,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34638,7 +34638,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34752,7 +34752,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34866,7 +34866,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34980,7 +34980,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35094,7 +35094,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35208,7 +35208,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35322,7 +35322,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35436,7 +35436,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35550,7 +35550,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:16 PM PT</t>
+          <t>2026-07-11 08:23:16 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35664,7 +35664,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35677,25 +35677,25 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F306" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H306" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I306" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J306" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K306" t="inlineStr">
         <is>
@@ -35787,7 +35787,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35901,7 +35901,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36015,7 +36015,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36129,7 +36129,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36243,7 +36243,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36357,7 +36357,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36471,7 +36471,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36585,7 +36585,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36699,7 +36699,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36813,7 +36813,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36927,7 +36927,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37041,7 +37041,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37155,7 +37155,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37269,7 +37269,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37383,7 +37383,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37497,7 +37497,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37611,7 +37611,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37725,7 +37725,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37839,7 +37839,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37953,7 +37953,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -38067,7 +38067,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:18 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38080,25 +38080,25 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Bottom 7 | 3 out</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F327" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H327" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J327" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K327" t="inlineStr">
         <is>
@@ -38190,68 +38190,77 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:18 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
-        <v>822711</v>
+        <v>823276</v>
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>1:05 PM PT</t>
+          <t>5:40 PM PT</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Final</t>
+          <t>Top 8 | 0 out</t>
         </is>
       </c>
       <c r="F328" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>Bottom</t>
-        </is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="H328" t="n">
+        <v>0</v>
+      </c>
+      <c r="I328" t="n">
+        <v>0</v>
+      </c>
+      <c r="J328" t="n">
+        <v>0</v>
       </c>
       <c r="K328" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Away</t>
         </is>
       </c>
       <c r="L328" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="M328" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="N328" t="inlineStr">
         <is>
-          <t>Daylen Lile</t>
+          <t>Luis Urías</t>
         </is>
       </c>
       <c r="O328" t="n">
-        <v>695734</v>
+        <v>649966</v>
       </c>
       <c r="P328" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>PH</t>
         </is>
       </c>
       <c r="Q328" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8 (Sub)</t>
         </is>
       </c>
       <c r="R328" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S328" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="T328" t="n">
         <v>0</v>
@@ -38284,16 +38293,16 @@
         <v>0</v>
       </c>
       <c r="AD328" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE328" s="4" t="n">
         <v>0</v>
       </c>
       <c r="AF328" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AG328" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="329">
@@ -38304,7 +38313,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:21:17 PM PT</t>
+          <t>2026-07-11 08:23:17 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38345,27 +38354,27 @@
       </c>
       <c r="N329" t="inlineStr">
         <is>
-          <t>José Tena</t>
+          <t>Daylen Lile</t>
         </is>
       </c>
       <c r="O329" t="n">
-        <v>677588</v>
+        <v>695734</v>
       </c>
       <c r="P329" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="Q329" t="inlineStr">
         <is>
-          <t>8 (Sub)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R329" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S329" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T329" t="n">
         <v>0</v>
@@ -38398,7 +38407,7 @@
         <v>0</v>
       </c>
       <c r="AD329" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE329" s="4" t="n">
         <v>0</v>
@@ -38410,9 +38419,123 @@
         <v>7</v>
       </c>
     </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>2026-07-11 08:23:17 PM PT</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>822711</v>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>1:05 PM PT</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>9</v>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>NYY</t>
+        </is>
+      </c>
+      <c r="N330" t="inlineStr">
+        <is>
+          <t>José Tena</t>
+        </is>
+      </c>
+      <c r="O330" t="n">
+        <v>677588</v>
+      </c>
+      <c r="P330" t="inlineStr">
+        <is>
+          <t>PH</t>
+        </is>
+      </c>
+      <c r="Q330" t="inlineStr">
+        <is>
+          <t>8 (Sub)</t>
+        </is>
+      </c>
+      <c r="R330" t="n">
+        <v>1</v>
+      </c>
+      <c r="S330" t="n">
+        <v>1</v>
+      </c>
+      <c r="T330" t="n">
+        <v>0</v>
+      </c>
+      <c r="U330" t="n">
+        <v>0</v>
+      </c>
+      <c r="V330" t="n">
+        <v>0</v>
+      </c>
+      <c r="W330" t="n">
+        <v>0</v>
+      </c>
+      <c r="X330" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y330" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z330" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA330" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB330" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC330" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD330" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE330" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF330" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG330" t="n">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AG329"/>
-  <conditionalFormatting sqref="AE2:AE329">
+  <autoFilter ref="A1:AG330"/>
+  <conditionalFormatting sqref="AE2:AE330">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:25:19 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -487,7 +487,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -949,10 +949,10 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1642,10 +1642,10 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1993,10 +1993,10 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2458,10 +2458,10 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -3030,17 +3030,17 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4500,7 +4500,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4642,10 +4642,10 @@
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -5214,17 +5214,17 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6355,7 +6355,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -6363,17 +6363,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6579,7 +6579,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6807,7 +6807,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7035,7 +7035,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7377,7 +7377,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7605,7 +7605,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7719,7 +7719,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7747,10 +7747,10 @@
         <v>0</v>
       </c>
       <c r="I63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -7842,7 +7842,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -7863,17 +7863,17 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H64" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8193,7 +8193,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8221,10 +8221,10 @@
         <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8316,7 +8316,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8430,7 +8430,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -8679,17 +8679,17 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H71" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -8781,7 +8781,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -9009,7 +9009,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9123,7 +9123,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9151,10 +9151,10 @@
         <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J75" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9702,7 +9702,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10272,7 +10272,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10386,7 +10386,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10500,7 +10500,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10728,7 +10728,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10756,10 +10756,10 @@
         <v>0</v>
       </c>
       <c r="I89" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J89" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11092,7 +11092,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -11100,17 +11100,17 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H92" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11316,7 +11316,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11430,7 +11430,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11544,7 +11544,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11772,7 +11772,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11785,7 +11785,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -11793,17 +11793,17 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H98" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -11895,7 +11895,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12123,7 +12123,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12351,7 +12351,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12379,10 +12379,10 @@
         <v>0</v>
       </c>
       <c r="I103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J103" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12588,7 +12588,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12702,7 +12702,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12816,7 +12816,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12930,7 +12930,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13044,7 +13044,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13158,7 +13158,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13386,7 +13386,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13614,7 +13614,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13728,7 +13728,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13756,10 +13756,10 @@
         <v>0</v>
       </c>
       <c r="I115" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J115" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -13851,7 +13851,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13965,7 +13965,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14193,7 +14193,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14307,7 +14307,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14535,7 +14535,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14649,7 +14649,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14763,7 +14763,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14877,7 +14877,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15105,7 +15105,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15219,7 +15219,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15232,7 +15232,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -15240,17 +15240,17 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H128" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J128" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15342,7 +15342,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15456,7 +15456,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15570,7 +15570,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15684,7 +15684,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15912,7 +15912,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16026,7 +16026,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16140,7 +16140,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16368,7 +16368,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16482,7 +16482,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16596,7 +16596,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16824,7 +16824,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16938,7 +16938,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17052,7 +17052,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17166,7 +17166,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17280,7 +17280,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17293,7 +17293,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -17301,17 +17301,17 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H146" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J146" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K146" t="inlineStr">
         <is>
@@ -17403,7 +17403,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17517,7 +17517,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17745,7 +17745,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17973,7 +17973,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18087,7 +18087,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18315,7 +18315,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18429,7 +18429,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18457,10 +18457,10 @@
         <v>0</v>
       </c>
       <c r="I156" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J156" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -18552,7 +18552,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18580,10 +18580,10 @@
         <v>0</v>
       </c>
       <c r="I157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J157" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -18675,7 +18675,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18703,10 +18703,10 @@
         <v>0</v>
       </c>
       <c r="I158" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J158" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18826,10 +18826,10 @@
         <v>0</v>
       </c>
       <c r="I159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J159" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19263,7 +19263,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19377,7 +19377,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19605,7 +19605,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20175,7 +20175,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20188,7 +20188,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -20196,17 +20196,17 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H171" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J171" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20298,7 +20298,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20311,7 +20311,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20319,17 +20319,17 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H172" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J172" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20421,7 +20421,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20763,7 +20763,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20877,7 +20877,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20991,7 +20991,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21105,7 +21105,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21333,7 +21333,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21561,7 +21561,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21789,7 +21789,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21903,7 +21903,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22017,7 +22017,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22131,7 +22131,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22245,7 +22245,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22473,7 +22473,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22587,7 +22587,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22600,7 +22600,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -22608,17 +22608,17 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H192" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J192" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K192" t="inlineStr">
         <is>
@@ -22710,7 +22710,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22723,7 +22723,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -22731,17 +22731,17 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H193" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I193" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J193" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K193" t="inlineStr">
         <is>
@@ -22833,7 +22833,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22947,7 +22947,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23061,7 +23061,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23175,7 +23175,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23289,7 +23289,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23403,7 +23403,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23517,7 +23517,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23631,7 +23631,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23745,7 +23745,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23859,7 +23859,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23973,7 +23973,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24087,7 +24087,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24201,7 +24201,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24429,7 +24429,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24543,7 +24543,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24657,7 +24657,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24771,7 +24771,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24885,7 +24885,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24999,7 +24999,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25113,7 +25113,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25227,7 +25227,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25341,7 +25341,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25455,7 +25455,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25569,7 +25569,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25683,7 +25683,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25797,7 +25797,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25911,7 +25911,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26025,7 +26025,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26139,7 +26139,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26253,7 +26253,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26367,7 +26367,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26481,7 +26481,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26595,7 +26595,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26709,7 +26709,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26823,7 +26823,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26851,10 +26851,10 @@
         <v>0</v>
       </c>
       <c r="I229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J229" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K229" t="inlineStr">
         <is>
@@ -26946,7 +26946,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27060,7 +27060,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27174,7 +27174,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27288,7 +27288,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27402,7 +27402,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27415,7 +27415,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F234" t="n">
@@ -27423,17 +27423,17 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H234" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I234" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J234" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K234" t="inlineStr">
         <is>
@@ -27525,7 +27525,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27538,7 +27538,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F235" t="n">
@@ -27546,17 +27546,17 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H235" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J235" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K235" t="inlineStr">
         <is>
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27762,7 +27762,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27876,7 +27876,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27990,7 +27990,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28104,7 +28104,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28218,7 +28218,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28332,7 +28332,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28446,7 +28446,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28560,7 +28560,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28674,7 +28674,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28788,7 +28788,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28902,7 +28902,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29016,7 +29016,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29130,7 +29130,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29244,7 +29244,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29472,7 +29472,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29586,7 +29586,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29700,7 +29700,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29814,7 +29814,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29928,7 +29928,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30042,7 +30042,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30156,7 +30156,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30270,7 +30270,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30384,7 +30384,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30498,7 +30498,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30612,7 +30612,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30726,7 +30726,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30840,7 +30840,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30954,7 +30954,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31068,7 +31068,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31182,7 +31182,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31296,7 +31296,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31410,7 +31410,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31524,7 +31524,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31638,7 +31638,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31752,7 +31752,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31866,7 +31866,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31980,7 +31980,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32094,7 +32094,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32208,7 +32208,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32322,7 +32322,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32436,7 +32436,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32449,7 +32449,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F278" t="n">
@@ -32457,17 +32457,17 @@
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H278" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I278" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J278" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K278" t="inlineStr">
         <is>
@@ -32559,7 +32559,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32572,7 +32572,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F279" t="n">
@@ -32580,17 +32580,17 @@
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H279" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I279" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J279" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K279" t="inlineStr">
         <is>
@@ -32682,7 +32682,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32695,7 +32695,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F280" t="n">
@@ -32703,17 +32703,17 @@
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H280" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I280" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J280" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K280" t="inlineStr">
         <is>
@@ -32805,7 +32805,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32818,7 +32818,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Top 7 | 3 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -32826,17 +32826,17 @@
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H281" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I281" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J281" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K281" t="inlineStr">
         <is>
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33042,7 +33042,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33156,7 +33156,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33270,7 +33270,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33384,7 +33384,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33498,7 +33498,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33612,7 +33612,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33726,7 +33726,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33840,7 +33840,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33954,7 +33954,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34068,7 +34068,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34182,7 +34182,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34296,7 +34296,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34410,7 +34410,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34524,7 +34524,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34638,7 +34638,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34752,7 +34752,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34866,7 +34866,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34980,7 +34980,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35094,7 +35094,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35208,7 +35208,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35322,7 +35322,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35436,7 +35436,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35550,7 +35550,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:16 PM PT</t>
+          <t>2026-07-11 08:25:16 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35664,7 +35664,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35692,10 +35692,10 @@
         <v>0</v>
       </c>
       <c r="I306" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J306" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K306" t="inlineStr">
         <is>
@@ -35787,7 +35787,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35901,7 +35901,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36015,7 +36015,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36129,7 +36129,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36243,7 +36243,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36357,7 +36357,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36471,7 +36471,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36585,7 +36585,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36699,7 +36699,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36813,7 +36813,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36927,7 +36927,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37041,7 +37041,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37155,7 +37155,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37269,7 +37269,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37383,7 +37383,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37497,7 +37497,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37611,7 +37611,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37725,7 +37725,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37839,7 +37839,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37953,7 +37953,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -38067,7 +38067,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38095,10 +38095,10 @@
         <v>0</v>
       </c>
       <c r="I327" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J327" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K327" t="inlineStr">
         <is>
@@ -38190,7 +38190,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:18 PM PT</t>
+          <t>2026-07-11 08:25:18 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38218,10 +38218,10 @@
         <v>0</v>
       </c>
       <c r="I328" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J328" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K328" t="inlineStr">
         <is>
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:23:17 PM PT</t>
+          <t>2026-07-11 08:25:17 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:29:19 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -934,7 +934,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -946,13 +946,13 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -1639,13 +1639,13 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1990,13 +1990,13 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -2032,10 +2032,10 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T13" t="n">
         <v>1</v>
@@ -2068,7 +2068,7 @@
         <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE13" s="4" t="n">
         <v>22</v>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -2455,13 +2455,13 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -3034,13 +3034,13 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4044,7 +4044,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4500,7 +4500,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -4639,13 +4639,13 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -5218,13 +5218,13 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5430,7 +5430,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6342,7 +6342,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6355,7 +6355,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -6367,13 +6367,13 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6579,7 +6579,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6807,7 +6807,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7035,7 +7035,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7149,7 +7149,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7377,7 +7377,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7491,7 +7491,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7605,7 +7605,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7719,7 +7719,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7732,7 +7732,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -7744,13 +7744,13 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -7842,7 +7842,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F64" t="n">
@@ -7867,13 +7867,13 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K64" t="inlineStr">
         <is>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8193,7 +8193,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8206,7 +8206,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -8218,13 +8218,13 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8316,7 +8316,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8430,7 +8430,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -8683,13 +8683,13 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -8781,7 +8781,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8895,7 +8895,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -9009,7 +9009,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9123,7 +9123,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9136,7 +9136,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F75" t="n">
@@ -9148,13 +9148,13 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J75" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -9190,10 +9190,10 @@
         </is>
       </c>
       <c r="R75" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T75" t="n">
         <v>1</v>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9360,7 +9360,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9588,7 +9588,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9702,7 +9702,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9930,7 +9930,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10158,7 +10158,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10272,7 +10272,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10386,7 +10386,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10500,7 +10500,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10614,7 +10614,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10728,7 +10728,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10741,7 +10741,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -10753,13 +10753,13 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11092,7 +11092,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -11104,13 +11104,13 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J92" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -11202,7 +11202,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11316,7 +11316,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11430,7 +11430,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11544,7 +11544,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11772,7 +11772,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11785,7 +11785,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -11797,13 +11797,13 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J98" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -11839,10 +11839,10 @@
         </is>
       </c>
       <c r="R98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T98" t="n">
         <v>1</v>
@@ -11895,7 +11895,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12123,7 +12123,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12351,7 +12351,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12364,7 +12364,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -12376,13 +12376,13 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J103" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12588,7 +12588,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12702,7 +12702,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12816,7 +12816,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12930,7 +12930,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13044,7 +13044,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13158,7 +13158,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13386,7 +13386,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13614,7 +13614,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13728,7 +13728,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13741,7 +13741,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F115" t="n">
@@ -13753,13 +13753,13 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I115" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J115" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K115" t="inlineStr">
         <is>
@@ -13851,7 +13851,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13965,7 +13965,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14193,7 +14193,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14307,7 +14307,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14535,7 +14535,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14649,7 +14649,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14763,7 +14763,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14877,7 +14877,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15105,7 +15105,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15219,7 +15219,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15232,7 +15232,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -15244,13 +15244,13 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I128" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J128" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15342,7 +15342,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15456,7 +15456,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15570,7 +15570,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15684,7 +15684,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15912,7 +15912,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16026,7 +16026,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16140,7 +16140,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16368,7 +16368,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16482,7 +16482,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16596,7 +16596,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16824,7 +16824,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16938,7 +16938,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17052,7 +17052,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17166,7 +17166,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17280,7 +17280,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17293,7 +17293,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -17305,13 +17305,13 @@
         </is>
       </c>
       <c r="H146" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I146" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K146" t="inlineStr">
         <is>
@@ -17403,7 +17403,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17517,7 +17517,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17745,7 +17745,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17973,7 +17973,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18087,7 +18087,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18315,7 +18315,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18429,7 +18429,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18442,7 +18442,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F156" t="n">
@@ -18454,13 +18454,13 @@
         </is>
       </c>
       <c r="H156" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I156" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J156" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -18552,7 +18552,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18565,7 +18565,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F157" t="n">
@@ -18577,13 +18577,13 @@
         </is>
       </c>
       <c r="H157" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J157" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -18675,7 +18675,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -18700,13 +18700,13 @@
         </is>
       </c>
       <c r="H158" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I158" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J158" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18811,7 +18811,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -18823,13 +18823,13 @@
         </is>
       </c>
       <c r="H159" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J159" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19263,7 +19263,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19377,7 +19377,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19605,7 +19605,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20175,7 +20175,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20188,7 +20188,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -20200,13 +20200,13 @@
         </is>
       </c>
       <c r="H171" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I171" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J171" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20298,7 +20298,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20311,7 +20311,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20323,13 +20323,13 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I172" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J172" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20421,7 +20421,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20763,7 +20763,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20877,7 +20877,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20991,7 +20991,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21105,7 +21105,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21333,7 +21333,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21561,7 +21561,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21789,7 +21789,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21903,7 +21903,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22017,7 +22017,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22131,7 +22131,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22245,7 +22245,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22372,7 +22372,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -22384,13 +22384,13 @@
         </is>
       </c>
       <c r="H190" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I190" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J190" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
@@ -22482,7 +22482,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22596,7 +22596,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22710,7 +22710,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22723,7 +22723,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -22735,13 +22735,13 @@
         </is>
       </c>
       <c r="H193" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I193" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J193" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K193" t="inlineStr">
         <is>
@@ -22833,7 +22833,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22846,7 +22846,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -22858,13 +22858,13 @@
         </is>
       </c>
       <c r="H194" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I194" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J194" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K194" t="inlineStr">
         <is>
@@ -22956,7 +22956,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23070,7 +23070,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23184,7 +23184,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23298,7 +23298,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23412,7 +23412,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23526,7 +23526,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23640,7 +23640,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23754,7 +23754,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23868,7 +23868,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23982,7 +23982,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24210,7 +24210,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24324,7 +24324,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24438,7 +24438,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24552,7 +24552,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24666,7 +24666,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24780,7 +24780,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24894,7 +24894,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25008,7 +25008,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25122,7 +25122,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25236,7 +25236,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25350,7 +25350,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25464,7 +25464,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25578,7 +25578,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25692,7 +25692,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25806,7 +25806,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25920,7 +25920,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26034,7 +26034,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26148,7 +26148,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26262,7 +26262,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26376,7 +26376,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26490,7 +26490,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26604,7 +26604,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26718,7 +26718,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26832,7 +26832,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26946,7 +26946,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26959,7 +26959,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -26971,13 +26971,13 @@
         </is>
       </c>
       <c r="H230" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I230" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J230" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K230" t="inlineStr">
         <is>
@@ -27069,7 +27069,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27183,7 +27183,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27297,7 +27297,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27411,7 +27411,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27525,7 +27525,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27538,7 +27538,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F235" t="n">
@@ -27550,13 +27550,13 @@
         </is>
       </c>
       <c r="H235" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I235" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J235" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K235" t="inlineStr">
         <is>
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27661,7 +27661,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -27673,13 +27673,13 @@
         </is>
       </c>
       <c r="H236" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I236" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J236" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K236" t="inlineStr">
         <is>
@@ -27771,7 +27771,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27885,7 +27885,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27999,7 +27999,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28113,7 +28113,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28227,7 +28227,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28341,7 +28341,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28455,7 +28455,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28569,7 +28569,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28683,7 +28683,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28797,7 +28797,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28911,7 +28911,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29025,7 +29025,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29139,7 +29139,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29253,7 +29253,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29367,7 +29367,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29481,7 +29481,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29595,7 +29595,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29709,7 +29709,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29823,7 +29823,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29937,7 +29937,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30051,7 +30051,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30165,7 +30165,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30279,7 +30279,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30393,7 +30393,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30507,7 +30507,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30621,7 +30621,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30735,7 +30735,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30849,7 +30849,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30963,7 +30963,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31191,7 +31191,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31305,7 +31305,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31419,7 +31419,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31533,7 +31533,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31647,7 +31647,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31761,7 +31761,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31875,7 +31875,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31989,7 +31989,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32103,7 +32103,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32217,7 +32217,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32331,7 +32331,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32445,7 +32445,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32559,7 +32559,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32572,7 +32572,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F279" t="n">
@@ -32584,13 +32584,13 @@
         </is>
       </c>
       <c r="H279" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I279" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J279" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K279" t="inlineStr">
         <is>
@@ -32682,7 +32682,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32695,7 +32695,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F280" t="n">
@@ -32707,13 +32707,13 @@
         </is>
       </c>
       <c r="H280" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I280" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J280" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K280" t="inlineStr">
         <is>
@@ -32805,7 +32805,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32818,7 +32818,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -32830,13 +32830,13 @@
         </is>
       </c>
       <c r="H281" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I281" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J281" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K281" t="inlineStr">
         <is>
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32941,7 +32941,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Bottom 7 | 1 out</t>
+          <t>Bottom 7 | 3 out</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -32953,13 +32953,13 @@
         </is>
       </c>
       <c r="H282" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I282" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J282" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K282" t="inlineStr">
         <is>
@@ -32995,10 +32995,10 @@
         </is>
       </c>
       <c r="R282" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S282" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T282" t="n">
         <v>0</v>
@@ -33051,7 +33051,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33165,7 +33165,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33279,7 +33279,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33393,7 +33393,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33507,7 +33507,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33621,7 +33621,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33735,7 +33735,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33849,7 +33849,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33963,7 +33963,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34077,7 +34077,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34191,7 +34191,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34305,7 +34305,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34419,7 +34419,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34533,7 +34533,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34647,7 +34647,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34761,7 +34761,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34875,7 +34875,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34989,7 +34989,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35103,7 +35103,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35217,7 +35217,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35331,7 +35331,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35445,7 +35445,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35559,7 +35559,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35673,7 +35673,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:16 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35787,7 +35787,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35800,7 +35800,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F307" t="n">
@@ -35812,13 +35812,13 @@
         </is>
       </c>
       <c r="H307" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I307" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J307" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K307" t="inlineStr">
         <is>
@@ -35910,7 +35910,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36024,7 +36024,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36138,7 +36138,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36252,7 +36252,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36366,7 +36366,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36480,7 +36480,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36594,7 +36594,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:16 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36708,7 +36708,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36822,7 +36822,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36936,7 +36936,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37050,7 +37050,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37164,7 +37164,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37278,7 +37278,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37392,7 +37392,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37506,7 +37506,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37620,7 +37620,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37734,7 +37734,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37848,7 +37848,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37962,7 +37962,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -38076,7 +38076,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38190,7 +38190,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:18 PM PT</t>
+          <t>2026-07-11 08:29:18 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38203,7 +38203,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 3 out</t>
         </is>
       </c>
       <c r="F328" t="n">
@@ -38215,13 +38215,13 @@
         </is>
       </c>
       <c r="H328" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I328" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J328" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K328" t="inlineStr">
         <is>
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:27:17 PM PT</t>
+          <t>2026-07-11 08:29:17 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:33:55 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -835,7 +835,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
@@ -930,7 +930,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3160,7 +3160,7 @@
         <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J23" t="n">
         <v>1</v>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4623,7 +4623,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4860,7 +4860,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4974,7 +4974,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5344,7 +5344,7 @@
         <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J42" t="n">
         <v>1</v>
@@ -5439,7 +5439,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5895,7 +5895,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6616,7 +6616,7 @@
         <v>1</v>
       </c>
       <c r="I53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J53" t="n">
         <v>1</v>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6825,7 +6825,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7053,7 +7053,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7737,7 +7737,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7965,7 +7965,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8088,7 +8088,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8116,7 +8116,7 @@
         <v>1</v>
       </c>
       <c r="I66" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J66" t="n">
         <v>1</v>
@@ -8211,7 +8211,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8439,7 +8439,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8553,7 +8553,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8667,7 +8667,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8781,7 +8781,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8809,7 +8809,7 @@
         <v>1</v>
       </c>
       <c r="I72" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J72" t="n">
         <v>1</v>
@@ -8904,7 +8904,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9132,7 +9132,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9246,7 +9246,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9369,7 +9369,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10053,7 +10053,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10974,7 +10974,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11202,7 +11202,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11230,7 +11230,7 @@
         <v>1</v>
       </c>
       <c r="I93" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J93" t="n">
         <v>1</v>
@@ -11325,7 +11325,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11439,7 +11439,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11553,7 +11553,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11667,7 +11667,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11781,7 +11781,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11923,7 +11923,7 @@
         <v>1</v>
       </c>
       <c r="I99" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J99" t="n">
         <v>1</v>
@@ -12018,7 +12018,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12246,7 +12246,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12360,7 +12360,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12474,7 +12474,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12711,7 +12711,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12825,7 +12825,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12939,7 +12939,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13053,7 +13053,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13167,7 +13167,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13281,7 +13281,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13395,7 +13395,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13509,7 +13509,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13851,7 +13851,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13974,7 +13974,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14202,7 +14202,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14316,7 +14316,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14430,7 +14430,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14658,7 +14658,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14772,7 +14772,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14886,7 +14886,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -15000,7 +15000,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15114,7 +15114,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15342,7 +15342,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15370,7 +15370,7 @@
         <v>1</v>
       </c>
       <c r="I129" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J129" t="n">
         <v>1</v>
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15579,7 +15579,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15693,7 +15693,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15807,7 +15807,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16035,7 +16035,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16149,7 +16149,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16263,7 +16263,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16377,7 +16377,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16491,7 +16491,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16605,7 +16605,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16719,7 +16719,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16833,7 +16833,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16947,7 +16947,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17061,7 +17061,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17175,7 +17175,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17289,7 +17289,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17403,7 +17403,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17517,7 +17517,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17745,7 +17745,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17973,7 +17973,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18087,7 +18087,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18315,7 +18315,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18429,7 +18429,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18552,7 +18552,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18675,7 +18675,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19263,7 +19263,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19377,7 +19377,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19605,7 +19605,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20175,7 +20175,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20203,7 +20203,7 @@
         <v>1</v>
       </c>
       <c r="I171" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J171" t="n">
         <v>1</v>
@@ -20298,7 +20298,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20326,7 +20326,7 @@
         <v>1</v>
       </c>
       <c r="I172" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J172" t="n">
         <v>1</v>
@@ -20421,7 +20421,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20763,7 +20763,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20877,7 +20877,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20991,7 +20991,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21105,7 +21105,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21333,7 +21333,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21561,7 +21561,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21789,7 +21789,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21903,7 +21903,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22017,7 +22017,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22131,7 +22131,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22245,7 +22245,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22482,7 +22482,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22596,7 +22596,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22710,7 +22710,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22738,7 +22738,7 @@
         <v>1</v>
       </c>
       <c r="I193" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J193" t="n">
         <v>1</v>
@@ -22833,7 +22833,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22861,7 +22861,7 @@
         <v>1</v>
       </c>
       <c r="I194" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J194" t="n">
         <v>1</v>
@@ -22956,7 +22956,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23070,7 +23070,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23184,7 +23184,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23298,7 +23298,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23412,7 +23412,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23526,7 +23526,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23640,7 +23640,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23754,7 +23754,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23868,7 +23868,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23982,7 +23982,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24210,7 +24210,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24324,7 +24324,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24438,7 +24438,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24552,7 +24552,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24666,7 +24666,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24780,7 +24780,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24894,7 +24894,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25008,7 +25008,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25122,7 +25122,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25236,7 +25236,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25350,7 +25350,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25464,7 +25464,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25578,7 +25578,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25692,7 +25692,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25806,7 +25806,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25920,7 +25920,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26034,7 +26034,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26148,7 +26148,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26262,7 +26262,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26376,7 +26376,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26490,7 +26490,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26604,7 +26604,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26718,7 +26718,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26832,7 +26832,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26946,7 +26946,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27069,7 +27069,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27183,7 +27183,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27297,7 +27297,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27411,7 +27411,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27525,7 +27525,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27553,7 +27553,7 @@
         <v>1</v>
       </c>
       <c r="I235" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J235" t="n">
         <v>1</v>
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27676,7 +27676,7 @@
         <v>1</v>
       </c>
       <c r="I236" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J236" t="n">
         <v>1</v>
@@ -27771,7 +27771,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27885,7 +27885,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27999,7 +27999,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28113,7 +28113,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28227,7 +28227,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28341,7 +28341,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28455,7 +28455,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28569,7 +28569,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28683,7 +28683,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28797,7 +28797,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28911,7 +28911,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29025,7 +29025,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29139,7 +29139,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29253,7 +29253,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29367,7 +29367,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29481,7 +29481,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29595,7 +29595,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29709,7 +29709,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29823,7 +29823,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29937,7 +29937,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30051,7 +30051,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30165,7 +30165,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30279,7 +30279,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30393,7 +30393,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30507,7 +30507,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30621,7 +30621,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30735,7 +30735,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30849,7 +30849,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30963,7 +30963,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31191,7 +31191,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31305,7 +31305,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31419,7 +31419,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31533,7 +31533,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31647,7 +31647,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31761,7 +31761,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31875,7 +31875,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31989,7 +31989,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32103,7 +32103,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32217,7 +32217,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32331,7 +32331,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32445,7 +32445,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32559,7 +32559,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32587,7 +32587,7 @@
         <v>1</v>
       </c>
       <c r="I279" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J279" t="n">
         <v>1</v>
@@ -32682,7 +32682,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32710,7 +32710,7 @@
         <v>1</v>
       </c>
       <c r="I280" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J280" t="n">
         <v>1</v>
@@ -32805,7 +32805,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32833,7 +32833,7 @@
         <v>1</v>
       </c>
       <c r="I281" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J281" t="n">
         <v>1</v>
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32956,7 +32956,7 @@
         <v>1</v>
       </c>
       <c r="I282" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J282" t="n">
         <v>1</v>
@@ -33051,7 +33051,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33079,7 +33079,7 @@
         <v>1</v>
       </c>
       <c r="I283" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J283" t="n">
         <v>1</v>
@@ -33174,7 +33174,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33202,7 +33202,7 @@
         <v>1</v>
       </c>
       <c r="I284" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J284" t="n">
         <v>1</v>
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33325,7 +33325,7 @@
         <v>1</v>
       </c>
       <c r="I285" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J285" t="n">
         <v>1</v>
@@ -33420,7 +33420,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33534,7 +33534,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33648,7 +33648,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33762,7 +33762,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33876,7 +33876,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33990,7 +33990,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34104,7 +34104,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34218,7 +34218,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34332,7 +34332,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34446,7 +34446,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34560,7 +34560,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34674,7 +34674,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34788,7 +34788,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34902,7 +34902,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -35016,7 +35016,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35130,7 +35130,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35244,7 +35244,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35358,7 +35358,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35472,7 +35472,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35586,7 +35586,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35700,7 +35700,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35814,7 +35814,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35928,7 +35928,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36042,7 +36042,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:16 PM PT</t>
+          <t>2026-07-11 08:33:52 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36156,7 +36156,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36279,7 +36279,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36393,7 +36393,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36507,7 +36507,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36621,7 +36621,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36735,7 +36735,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36849,7 +36849,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36963,7 +36963,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37077,7 +37077,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37191,7 +37191,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37305,7 +37305,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37419,7 +37419,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37533,7 +37533,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37647,7 +37647,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37761,7 +37761,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37875,7 +37875,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37989,7 +37989,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -38103,7 +38103,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38217,7 +38217,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38445,7 +38445,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38559,7 +38559,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:18 PM PT</t>
+          <t>2026-07-11 08:33:54 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38682,7 +38682,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38796,7 +38796,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:17 PM PT</t>
+          <t>2026-07-11 08:33:53 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:35:56 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -832,13 +832,13 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1069,10 +1069,10 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -1762,10 +1762,10 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -2113,10 +2113,10 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -2578,10 +2578,10 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3145,7 +3145,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -3157,13 +3157,13 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4623,7 +4623,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -4762,10 +4762,10 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4974,7 +4974,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -5341,13 +5341,13 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -5439,7 +5439,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5895,7 +5895,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6478,7 +6478,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -6490,10 +6490,10 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6601,7 +6601,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -6613,13 +6613,13 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6825,7 +6825,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7053,7 +7053,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7737,7 +7737,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7965,7 +7965,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7978,7 +7978,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -7990,10 +7990,10 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J65" t="n">
         <v>0</v>
@@ -8088,7 +8088,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8101,7 +8101,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -8113,13 +8113,13 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I66" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -8211,7 +8211,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8439,7 +8439,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8553,7 +8553,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8667,7 +8667,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8781,7 +8781,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8794,7 +8794,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8806,13 +8806,13 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I72" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -8904,7 +8904,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9132,7 +9132,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9246,7 +9246,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9259,7 +9259,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -9271,10 +9271,10 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J76" t="n">
         <v>0</v>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10053,7 +10053,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -10876,10 +10876,10 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J90" t="n">
         <v>0</v>
@@ -10974,7 +10974,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11202,7 +11202,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11215,7 +11215,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11227,13 +11227,13 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I93" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -11325,7 +11325,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11439,7 +11439,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11553,7 +11553,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11667,7 +11667,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11781,7 +11781,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11908,7 +11908,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11920,13 +11920,13 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I99" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -12018,7 +12018,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12246,7 +12246,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12360,7 +12360,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12474,7 +12474,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12487,7 +12487,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -12499,10 +12499,10 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J104" t="n">
         <v>0</v>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12711,7 +12711,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12825,7 +12825,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12939,7 +12939,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13053,7 +13053,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13167,7 +13167,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13281,7 +13281,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13395,7 +13395,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13509,7 +13509,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13851,7 +13851,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13864,7 +13864,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F116" t="n">
@@ -13876,10 +13876,10 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J116" t="n">
         <v>0</v>
@@ -13974,7 +13974,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14202,7 +14202,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14316,7 +14316,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14430,7 +14430,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14658,7 +14658,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14772,7 +14772,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14886,7 +14886,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -15000,7 +15000,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15114,7 +15114,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15342,7 +15342,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15355,7 +15355,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -15367,13 +15367,13 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I129" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15579,7 +15579,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15693,7 +15693,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15807,7 +15807,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16035,7 +16035,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16149,7 +16149,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16263,7 +16263,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16377,7 +16377,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16491,7 +16491,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16605,7 +16605,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16719,7 +16719,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16833,7 +16833,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16947,7 +16947,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17061,7 +17061,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17175,7 +17175,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17289,7 +17289,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17403,7 +17403,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17517,7 +17517,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17745,7 +17745,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17973,7 +17973,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18087,7 +18087,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18315,7 +18315,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18429,7 +18429,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18442,7 +18442,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F156" t="n">
@@ -18454,10 +18454,10 @@
         </is>
       </c>
       <c r="H156" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I156" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J156" t="n">
         <v>0</v>
@@ -18552,7 +18552,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18565,7 +18565,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F157" t="n">
@@ -18577,10 +18577,10 @@
         </is>
       </c>
       <c r="H157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I157" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J157" t="n">
         <v>0</v>
@@ -18675,7 +18675,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -18700,10 +18700,10 @@
         </is>
       </c>
       <c r="H158" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I158" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J158" t="n">
         <v>0</v>
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18811,7 +18811,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -18823,10 +18823,10 @@
         </is>
       </c>
       <c r="H159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I159" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J159" t="n">
         <v>0</v>
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19263,7 +19263,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19377,7 +19377,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19605,7 +19605,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20175,7 +20175,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20188,7 +20188,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -20200,13 +20200,13 @@
         </is>
       </c>
       <c r="H171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I171" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20298,7 +20298,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20311,7 +20311,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20323,13 +20323,13 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I172" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20421,7 +20421,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20763,7 +20763,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20877,7 +20877,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20991,7 +20991,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21105,7 +21105,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21333,7 +21333,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21561,7 +21561,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21789,7 +21789,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21903,7 +21903,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22017,7 +22017,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22131,7 +22131,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22245,7 +22245,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22372,7 +22372,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -22384,10 +22384,10 @@
         </is>
       </c>
       <c r="H190" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I190" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J190" t="n">
         <v>0</v>
@@ -22482,7 +22482,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22596,7 +22596,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22710,7 +22710,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22723,7 +22723,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -22735,13 +22735,13 @@
         </is>
       </c>
       <c r="H193" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I193" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J193" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K193" t="inlineStr">
         <is>
@@ -22833,7 +22833,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22846,7 +22846,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -22858,13 +22858,13 @@
         </is>
       </c>
       <c r="H194" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I194" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J194" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K194" t="inlineStr">
         <is>
@@ -22956,7 +22956,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23070,7 +23070,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23184,7 +23184,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23298,7 +23298,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23412,7 +23412,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23526,7 +23526,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23640,7 +23640,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23754,7 +23754,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23868,7 +23868,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23982,7 +23982,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24210,7 +24210,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24324,7 +24324,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24438,7 +24438,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24552,7 +24552,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24666,7 +24666,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24780,7 +24780,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24894,7 +24894,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25008,7 +25008,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25122,7 +25122,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25236,7 +25236,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25350,7 +25350,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25464,7 +25464,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25578,7 +25578,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25692,7 +25692,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25806,7 +25806,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25920,7 +25920,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26034,7 +26034,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26148,7 +26148,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26262,7 +26262,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26376,7 +26376,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26490,7 +26490,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26604,7 +26604,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26718,7 +26718,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26832,7 +26832,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26946,7 +26946,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26959,7 +26959,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -26971,10 +26971,10 @@
         </is>
       </c>
       <c r="H230" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I230" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J230" t="n">
         <v>0</v>
@@ -27069,7 +27069,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27183,7 +27183,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27297,7 +27297,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27411,7 +27411,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27525,7 +27525,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27538,7 +27538,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F235" t="n">
@@ -27550,13 +27550,13 @@
         </is>
       </c>
       <c r="H235" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I235" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J235" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K235" t="inlineStr">
         <is>
@@ -27592,10 +27592,10 @@
         </is>
       </c>
       <c r="R235" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S235" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T235" t="n">
         <v>0</v>
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27661,7 +27661,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -27673,13 +27673,13 @@
         </is>
       </c>
       <c r="H236" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I236" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J236" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K236" t="inlineStr">
         <is>
@@ -27771,7 +27771,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27885,7 +27885,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27999,7 +27999,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28113,7 +28113,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28227,7 +28227,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28341,7 +28341,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28455,7 +28455,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28569,7 +28569,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28683,7 +28683,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28797,7 +28797,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28911,7 +28911,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29025,7 +29025,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29139,7 +29139,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29253,7 +29253,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29367,7 +29367,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29481,7 +29481,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29595,7 +29595,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29709,7 +29709,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29823,7 +29823,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29937,7 +29937,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30051,7 +30051,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30165,7 +30165,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30279,7 +30279,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30393,7 +30393,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30507,7 +30507,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30621,7 +30621,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30735,7 +30735,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30849,7 +30849,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30963,7 +30963,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31191,7 +31191,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31305,7 +31305,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31419,7 +31419,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31533,7 +31533,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31647,7 +31647,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31761,7 +31761,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31875,7 +31875,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31989,7 +31989,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32103,7 +32103,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32217,7 +32217,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32331,7 +32331,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32445,7 +32445,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32559,7 +32559,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32572,7 +32572,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F279" t="n">
@@ -32584,13 +32584,13 @@
         </is>
       </c>
       <c r="H279" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I279" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J279" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K279" t="inlineStr">
         <is>
@@ -32682,7 +32682,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32695,7 +32695,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F280" t="n">
@@ -32707,13 +32707,13 @@
         </is>
       </c>
       <c r="H280" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I280" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J280" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K280" t="inlineStr">
         <is>
@@ -32805,7 +32805,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32818,7 +32818,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -32830,13 +32830,13 @@
         </is>
       </c>
       <c r="H281" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I281" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J281" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K281" t="inlineStr">
         <is>
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32941,7 +32941,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -32953,13 +32953,13 @@
         </is>
       </c>
       <c r="H282" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I282" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J282" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K282" t="inlineStr">
         <is>
@@ -33051,7 +33051,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33064,7 +33064,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F283" t="n">
@@ -33076,13 +33076,13 @@
         </is>
       </c>
       <c r="H283" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I283" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J283" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K283" t="inlineStr">
         <is>
@@ -33174,7 +33174,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33187,7 +33187,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F284" t="n">
@@ -33199,13 +33199,13 @@
         </is>
       </c>
       <c r="H284" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I284" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J284" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K284" t="inlineStr">
         <is>
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33310,7 +33310,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F285" t="n">
@@ -33322,13 +33322,13 @@
         </is>
       </c>
       <c r="H285" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I285" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J285" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K285" t="inlineStr">
         <is>
@@ -33420,7 +33420,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33534,7 +33534,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33648,7 +33648,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33762,7 +33762,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33876,7 +33876,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33990,7 +33990,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34104,7 +34104,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34218,7 +34218,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34332,7 +34332,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34446,7 +34446,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34560,7 +34560,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34674,7 +34674,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34788,7 +34788,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34902,7 +34902,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -35016,7 +35016,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35130,7 +35130,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35244,7 +35244,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35358,7 +35358,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35472,7 +35472,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35586,7 +35586,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35700,7 +35700,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35814,7 +35814,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35928,7 +35928,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36042,7 +36042,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:52 PM PT</t>
+          <t>2026-07-11 08:35:52 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36156,7 +36156,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36169,7 +36169,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F310" t="n">
@@ -36181,10 +36181,10 @@
         </is>
       </c>
       <c r="H310" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I310" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J310" t="n">
         <v>0</v>
@@ -36279,7 +36279,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36393,7 +36393,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36507,7 +36507,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36621,7 +36621,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36735,7 +36735,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36849,7 +36849,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36963,7 +36963,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37077,7 +37077,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37191,7 +37191,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37305,7 +37305,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37419,7 +37419,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37533,7 +37533,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37647,7 +37647,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37761,7 +37761,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37875,7 +37875,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37989,7 +37989,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -38103,7 +38103,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38217,7 +38217,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38331,7 +38331,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38445,7 +38445,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38559,7 +38559,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:54 PM PT</t>
+          <t>2026-07-11 08:35:54 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38572,7 +38572,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>Bottom 8 | 0 out</t>
+          <t>Bottom 8 | 1 out</t>
         </is>
       </c>
       <c r="F331" t="n">
@@ -38584,10 +38584,10 @@
         </is>
       </c>
       <c r="H331" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I331" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J331" t="n">
         <v>0</v>
@@ -38682,7 +38682,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38796,7 +38796,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 08:33:53 PM PT</t>
+          <t>2026-07-11 08:35:53 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:43:55 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -487,7 +487,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,25 +820,25 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1057,25 +1057,25 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1750,25 +1750,25 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2101,25 +2101,25 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2566,25 +2566,25 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3145,25 +3145,25 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3825,7 +3825,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4053,7 +4053,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4167,7 +4167,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4395,7 +4395,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4623,7 +4623,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4737,7 +4737,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4750,25 +4750,25 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
@@ -4860,7 +4860,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4974,7 +4974,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5329,25 +5329,25 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K42" t="inlineStr">
         <is>
@@ -5439,7 +5439,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5895,7 +5895,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6478,25 +6478,25 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6601,25 +6601,25 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6825,7 +6825,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6939,7 +6939,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7053,7 +7053,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7509,7 +7509,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7737,7 +7737,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7965,7 +7965,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7978,25 +7978,25 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H65" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J65" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -8088,7 +8088,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8101,25 +8101,25 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H66" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -8211,7 +8211,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8439,7 +8439,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8553,7 +8553,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8667,7 +8667,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8781,7 +8781,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8794,25 +8794,25 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -8904,7 +8904,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9132,7 +9132,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9246,7 +9246,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9259,25 +9259,25 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F76" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H76" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J76" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9382,25 +9382,25 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F77" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H77" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J77" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -9492,7 +9492,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9948,7 +9948,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10062,7 +10062,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10176,7 +10176,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10290,7 +10290,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10518,7 +10518,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10632,7 +10632,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10746,7 +10746,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10860,7 +10860,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10974,7 +10974,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11202,7 +11202,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11215,25 +11215,25 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H93" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J93" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -11325,7 +11325,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11439,7 +11439,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11553,7 +11553,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11667,7 +11667,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11781,7 +11781,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11908,25 +11908,25 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H99" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J99" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -12018,7 +12018,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12246,7 +12246,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12360,7 +12360,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12474,7 +12474,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12487,25 +12487,25 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F104" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H104" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J104" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
@@ -12597,7 +12597,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12711,7 +12711,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12825,7 +12825,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12939,7 +12939,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13053,7 +13053,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13167,7 +13167,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13281,7 +13281,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13395,7 +13395,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13509,7 +13509,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13851,7 +13851,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13864,25 +13864,25 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H116" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I116" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J116" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K116" t="inlineStr">
         <is>
@@ -13974,7 +13974,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13987,25 +13987,25 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H117" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I117" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J117" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
@@ -14097,7 +14097,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14211,7 +14211,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14439,7 +14439,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14553,7 +14553,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14667,7 +14667,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14781,7 +14781,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14895,7 +14895,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -15009,7 +15009,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15351,7 +15351,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15478,25 +15478,25 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F130" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H130" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -15588,7 +15588,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15702,7 +15702,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15816,7 +15816,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15930,7 +15930,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16044,7 +16044,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16158,7 +16158,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16272,7 +16272,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16386,7 +16386,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16500,7 +16500,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16614,7 +16614,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16728,7 +16728,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16842,7 +16842,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16956,7 +16956,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17070,7 +17070,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17184,7 +17184,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17298,7 +17298,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17412,7 +17412,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17526,7 +17526,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17640,7 +17640,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17754,7 +17754,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17868,7 +17868,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17982,7 +17982,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18096,7 +18096,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18324,7 +18324,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18552,7 +18552,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18565,25 +18565,25 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F157" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H157" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J157" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -18675,7 +18675,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18688,25 +18688,25 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F158" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H158" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I158" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J158" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18811,25 +18811,25 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F159" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H159" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J159" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19263,7 +19263,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19377,7 +19377,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19605,7 +19605,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19947,7 +19947,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20175,7 +20175,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20188,25 +20188,25 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F171" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H171" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I171" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J171" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20298,7 +20298,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20311,25 +20311,25 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F172" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H172" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I172" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J172" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20421,7 +20421,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20763,7 +20763,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20877,7 +20877,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20991,7 +20991,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21105,7 +21105,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21219,7 +21219,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21333,7 +21333,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21447,7 +21447,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21561,7 +21561,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21789,7 +21789,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21903,7 +21903,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22017,7 +22017,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22131,7 +22131,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22245,7 +22245,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22359,7 +22359,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22372,25 +22372,25 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F190" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H190" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I190" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J190" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
@@ -22482,7 +22482,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22596,7 +22596,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22710,7 +22710,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22723,25 +22723,25 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F193" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H193" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I193" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J193" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K193" t="inlineStr">
         <is>
@@ -22833,7 +22833,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22846,25 +22846,25 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F194" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H194" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I194" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J194" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K194" t="inlineStr">
         <is>
@@ -22956,7 +22956,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23070,7 +23070,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23184,7 +23184,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23298,7 +23298,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23412,7 +23412,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23526,7 +23526,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23640,7 +23640,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23754,7 +23754,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23868,7 +23868,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23982,7 +23982,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24096,7 +24096,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24210,7 +24210,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24324,7 +24324,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24438,7 +24438,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24552,7 +24552,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24666,7 +24666,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24780,7 +24780,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24894,7 +24894,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25008,7 +25008,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25122,7 +25122,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25236,7 +25236,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25350,7 +25350,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25464,7 +25464,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25578,7 +25578,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25692,7 +25692,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25806,7 +25806,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25920,7 +25920,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26034,7 +26034,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26148,7 +26148,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26262,7 +26262,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26376,7 +26376,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26490,7 +26490,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26604,7 +26604,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26718,7 +26718,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26832,7 +26832,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26946,7 +26946,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26959,25 +26959,25 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F230" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H230" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I230" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J230" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K230" t="inlineStr">
         <is>
@@ -27069,7 +27069,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27183,7 +27183,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27297,7 +27297,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27411,7 +27411,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27525,7 +27525,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27538,25 +27538,25 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F235" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H235" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I235" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J235" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K235" t="inlineStr">
         <is>
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27661,25 +27661,25 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F236" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H236" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I236" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J236" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K236" t="inlineStr">
         <is>
@@ -27771,7 +27771,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27885,7 +27885,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27999,7 +27999,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28113,7 +28113,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28227,7 +28227,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28341,7 +28341,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28455,7 +28455,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28569,7 +28569,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28683,7 +28683,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28797,7 +28797,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28911,7 +28911,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29025,7 +29025,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29139,7 +29139,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29253,7 +29253,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29367,7 +29367,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29481,7 +29481,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29595,7 +29595,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29709,7 +29709,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29823,7 +29823,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29937,7 +29937,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30051,7 +30051,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30165,7 +30165,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30279,7 +30279,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30393,7 +30393,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30507,7 +30507,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30621,7 +30621,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30735,7 +30735,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30849,7 +30849,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30963,7 +30963,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31191,7 +31191,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31305,7 +31305,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31419,7 +31419,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31533,7 +31533,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31647,7 +31647,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31761,7 +31761,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31875,7 +31875,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31989,7 +31989,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32103,7 +32103,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32217,7 +32217,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32331,7 +32331,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32445,7 +32445,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32559,7 +32559,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32572,25 +32572,25 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F279" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H279" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I279" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J279" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K279" t="inlineStr">
         <is>
@@ -32617,7 +32617,7 @@
       </c>
       <c r="P279" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>DH</t>
         </is>
       </c>
       <c r="Q279" t="inlineStr">
@@ -32682,7 +32682,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32695,25 +32695,25 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F280" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H280" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I280" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J280" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K280" t="inlineStr">
         <is>
@@ -32749,10 +32749,10 @@
         </is>
       </c>
       <c r="R280" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S280" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T280" t="n">
         <v>0</v>
@@ -32785,7 +32785,7 @@
         <v>0</v>
       </c>
       <c r="AD280" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE280" s="4" t="n">
         <v>0</v>
@@ -32805,7 +32805,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32818,25 +32818,25 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F281" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H281" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I281" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J281" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K281" t="inlineStr">
         <is>
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32941,25 +32941,25 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F282" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H282" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I282" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J282" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K282" t="inlineStr">
         <is>
@@ -33051,7 +33051,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33064,25 +33064,25 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F283" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H283" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I283" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J283" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K283" t="inlineStr">
         <is>
@@ -33174,7 +33174,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33187,25 +33187,25 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F284" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H284" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I284" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J284" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K284" t="inlineStr">
         <is>
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33310,25 +33310,25 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F285" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H285" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I285" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J285" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K285" t="inlineStr">
         <is>
@@ -33420,7 +33420,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33433,25 +33433,25 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F286" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H286" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I286" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J286" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K286" t="inlineStr">
         <is>
@@ -33543,7 +33543,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33657,7 +33657,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33771,7 +33771,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33885,7 +33885,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33999,7 +33999,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34113,7 +34113,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34227,7 +34227,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34341,7 +34341,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34455,7 +34455,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34569,7 +34569,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34683,7 +34683,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34797,7 +34797,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34911,7 +34911,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -35025,7 +35025,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35139,7 +35139,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35253,7 +35253,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35367,7 +35367,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35481,7 +35481,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35595,7 +35595,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35709,7 +35709,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35823,7 +35823,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35937,7 +35937,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36051,7 +36051,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:52 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36165,7 +36165,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:52 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36279,7 +36279,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36292,25 +36292,25 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F311" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H311" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J311" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K311" t="inlineStr">
         <is>
@@ -36337,7 +36337,7 @@
       </c>
       <c r="P311" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="Q311" t="inlineStr">
@@ -36402,7 +36402,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36415,25 +36415,25 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F312" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H312" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J312" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K312" t="inlineStr">
         <is>
@@ -36525,7 +36525,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36639,7 +36639,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36753,7 +36753,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36867,7 +36867,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36981,7 +36981,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37095,7 +37095,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37209,7 +37209,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37323,7 +37323,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37437,7 +37437,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37551,7 +37551,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37665,7 +37665,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37779,7 +37779,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37893,7 +37893,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -38007,7 +38007,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -38121,7 +38121,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38235,7 +38235,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38349,7 +38349,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38463,7 +38463,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38577,7 +38577,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38691,7 +38691,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38805,7 +38805,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:54 PM PT</t>
+          <t>2026-07-11 08:43:54 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38818,25 +38818,25 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F333" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H333" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I333" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J333" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K333" t="inlineStr">
         <is>
@@ -38928,7 +38928,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -39042,7 +39042,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 08:41:53 PM PT</t>
+          <t>2026-07-11 08:43:53 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:51:55 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
         <v>1</v>
@@ -930,7 +930,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1067,15 +1067,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H5" t="n">
-        <v>3</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>3</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1167,7 +1158,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1281,7 +1272,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1395,7 +1386,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1509,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1623,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1737,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1750,7 +1741,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -1760,15 +1751,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H11" t="n">
-        <v>3</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>3</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1860,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1974,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2088,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2101,7 +2083,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -2111,15 +2093,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H14" t="n">
-        <v>3</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>3</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -2211,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2325,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2439,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2553,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2566,7 +2539,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -2576,15 +2549,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H18" t="n">
-        <v>3</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="n">
-        <v>3</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -2676,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2790,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2803,7 +2767,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -2815,7 +2779,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I20" t="n">
         <v>1</v>
@@ -2913,7 +2877,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3027,7 +2991,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3141,7 +3105,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3255,7 +3219,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3268,7 +3232,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -3280,7 +3244,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I24" t="n">
         <v>1</v>
@@ -3378,7 +3342,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3492,7 +3456,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3606,7 +3570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3720,7 +3684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3834,7 +3798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3948,7 +3912,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4062,7 +4026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4176,7 +4140,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4290,7 +4254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4404,7 +4368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4518,7 +4482,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4632,7 +4596,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4746,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4860,7 +4824,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4873,7 +4837,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -4883,15 +4847,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H38" t="n">
-        <v>3</v>
-      </c>
-      <c r="I38" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" t="n">
-        <v>3</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -4983,7 +4938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5097,7 +5052,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5211,7 +5166,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5325,7 +5280,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5439,7 +5394,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5452,7 +5407,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -5464,7 +5419,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I43" t="n">
         <v>1</v>
@@ -5562,7 +5517,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5676,7 +5631,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5790,7 +5745,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5904,7 +5859,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6018,7 +5973,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6132,7 +6087,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6246,7 +6201,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6360,7 +6315,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6474,7 +6429,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6588,7 +6543,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6601,7 +6556,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -6611,15 +6566,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H53" t="n">
-        <v>3</v>
-      </c>
-      <c r="I53" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" t="n">
-        <v>3</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -6711,7 +6657,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6724,7 +6670,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -6736,7 +6682,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I54" t="n">
         <v>1</v>
@@ -6834,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6948,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7062,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7176,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7290,7 +7236,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7404,7 +7350,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7518,7 +7464,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7632,7 +7578,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7746,7 +7692,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7860,7 +7806,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7974,7 +7920,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8088,7 +8034,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8101,7 +8047,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -8111,15 +8057,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H66" t="n">
-        <v>3</v>
-      </c>
-      <c r="I66" t="n">
-        <v>0</v>
-      </c>
-      <c r="J66" t="n">
-        <v>3</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -8211,7 +8148,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8325,7 +8262,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8439,7 +8376,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8553,7 +8490,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8667,7 +8604,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8781,7 +8718,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8794,7 +8731,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8806,7 +8743,7 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I72" t="n">
         <v>1</v>
@@ -8904,7 +8841,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -9018,7 +8955,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9132,7 +9069,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9246,7 +9183,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9259,7 +9196,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -9269,15 +9206,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H76" t="n">
-        <v>3</v>
-      </c>
-      <c r="I76" t="n">
-        <v>0</v>
-      </c>
-      <c r="J76" t="n">
-        <v>3</v>
       </c>
       <c r="K76" t="inlineStr">
         <is>
@@ -9369,7 +9297,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9382,7 +9310,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F77" t="n">
@@ -9392,15 +9320,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H77" t="n">
-        <v>3</v>
-      </c>
-      <c r="I77" t="n">
-        <v>0</v>
-      </c>
-      <c r="J77" t="n">
-        <v>3</v>
       </c>
       <c r="K77" t="inlineStr">
         <is>
@@ -9492,7 +9411,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9606,7 +9525,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9720,7 +9639,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9834,7 +9753,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9948,7 +9867,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10062,7 +9981,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10176,7 +10095,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10290,7 +10209,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10404,7 +10323,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10518,7 +10437,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10632,7 +10551,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10746,7 +10665,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10860,7 +10779,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10974,7 +10893,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11088,7 +11007,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11202,7 +11121,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11215,7 +11134,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11227,7 +11146,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I93" t="n">
         <v>1</v>
@@ -11325,7 +11244,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11439,7 +11358,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11553,7 +11472,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11667,7 +11586,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11781,7 +11700,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11895,7 +11814,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11908,7 +11827,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11920,7 +11839,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I99" t="n">
         <v>1</v>
@@ -12018,7 +11937,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12132,7 +12051,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12246,7 +12165,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12360,7 +12279,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12474,7 +12393,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12487,7 +12406,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -12497,15 +12416,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H104" t="n">
-        <v>3</v>
-      </c>
-      <c r="I104" t="n">
-        <v>0</v>
-      </c>
-      <c r="J104" t="n">
-        <v>3</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
@@ -12597,7 +12507,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12711,7 +12621,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12825,7 +12735,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12939,7 +12849,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13053,7 +12963,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13167,7 +13077,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13281,7 +13191,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13294,7 +13204,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F111" t="n">
@@ -13304,15 +13214,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H111" t="n">
-        <v>3</v>
-      </c>
-      <c r="I111" t="n">
-        <v>0</v>
-      </c>
-      <c r="J111" t="n">
-        <v>3</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -13404,7 +13305,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13518,7 +13419,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13632,7 +13533,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13746,7 +13647,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13860,7 +13761,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13974,7 +13875,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13987,7 +13888,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -13997,15 +13898,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H117" t="n">
-        <v>3</v>
-      </c>
-      <c r="I117" t="n">
-        <v>0</v>
-      </c>
-      <c r="J117" t="n">
-        <v>3</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
@@ -14097,7 +13989,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14110,7 +14002,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F118" t="n">
@@ -14120,15 +14012,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H118" t="n">
-        <v>3</v>
-      </c>
-      <c r="I118" t="n">
-        <v>0</v>
-      </c>
-      <c r="J118" t="n">
-        <v>3</v>
       </c>
       <c r="K118" t="inlineStr">
         <is>
@@ -14220,7 +14103,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14334,7 +14217,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14448,7 +14331,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14562,7 +14445,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14676,7 +14559,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14790,7 +14673,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14904,7 +14787,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -15018,7 +14901,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15132,7 +15015,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15246,7 +15129,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15360,7 +15243,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15474,7 +15357,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15588,7 +15471,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15601,7 +15484,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -15613,7 +15496,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I131" t="n">
         <v>1</v>
@@ -15711,7 +15594,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15825,7 +15708,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15939,7 +15822,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16053,7 +15936,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16167,7 +16050,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16281,7 +16164,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16395,7 +16278,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16509,7 +16392,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16623,7 +16506,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16737,7 +16620,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16851,7 +16734,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16965,7 +16848,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17079,7 +16962,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17193,7 +17076,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17307,7 +17190,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17421,7 +17304,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17535,7 +17418,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17649,7 +17532,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17662,7 +17545,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F149" t="n">
@@ -17672,15 +17555,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H149" t="n">
-        <v>3</v>
-      </c>
-      <c r="I149" t="n">
-        <v>0</v>
-      </c>
-      <c r="J149" t="n">
-        <v>3</v>
       </c>
       <c r="K149" t="inlineStr">
         <is>
@@ -17772,7 +17646,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17886,7 +17760,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -18000,7 +17874,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18114,7 +17988,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18228,7 +18102,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18342,7 +18216,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18456,7 +18330,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18570,7 +18444,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18684,7 +18558,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18798,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18811,7 +18685,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -18821,15 +18695,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H159" t="n">
-        <v>3</v>
-      </c>
-      <c r="I159" t="n">
-        <v>0</v>
-      </c>
-      <c r="J159" t="n">
-        <v>3</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -18921,7 +18786,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18934,7 +18799,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -18944,15 +18809,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H160" t="n">
-        <v>3</v>
-      </c>
-      <c r="I160" t="n">
-        <v>0</v>
-      </c>
-      <c r="J160" t="n">
-        <v>3</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
@@ -19044,7 +18900,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19158,7 +19014,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19272,7 +19128,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19386,7 +19242,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19500,7 +19356,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19614,7 +19470,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19728,7 +19584,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19842,7 +19698,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19956,7 +19812,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20070,7 +19926,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20184,7 +20040,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20298,7 +20154,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20311,7 +20167,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20323,7 +20179,7 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I172" t="n">
         <v>1</v>
@@ -20421,7 +20277,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20434,7 +20290,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -20446,7 +20302,7 @@
         </is>
       </c>
       <c r="H173" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I173" t="n">
         <v>1</v>
@@ -20544,7 +20400,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20658,7 +20514,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20772,7 +20628,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20886,7 +20742,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -21000,7 +20856,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21114,7 +20970,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21228,7 +21084,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21342,7 +21198,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21456,7 +21312,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21570,7 +21426,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21684,7 +21540,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21798,7 +21654,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21912,7 +21768,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22026,7 +21882,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22140,7 +21996,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22254,7 +22110,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22368,7 +22224,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22482,7 +22338,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22495,7 +22351,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -22505,15 +22361,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H191" t="n">
-        <v>3</v>
-      </c>
-      <c r="I191" t="n">
-        <v>0</v>
-      </c>
-      <c r="J191" t="n">
-        <v>3</v>
       </c>
       <c r="K191" t="inlineStr">
         <is>
@@ -22605,7 +22452,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22719,7 +22566,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22833,7 +22680,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22846,7 +22693,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -22858,7 +22705,7 @@
         </is>
       </c>
       <c r="H194" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I194" t="n">
         <v>1</v>
@@ -22956,7 +22803,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22969,7 +22816,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -22981,7 +22828,7 @@
         </is>
       </c>
       <c r="H195" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I195" t="n">
         <v>1</v>
@@ -23079,7 +22926,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23193,7 +23040,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23307,7 +23154,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23421,7 +23268,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23535,7 +23382,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23649,7 +23496,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23763,7 +23610,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23877,7 +23724,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23991,7 +23838,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24105,7 +23952,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24219,7 +24066,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24333,7 +24180,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24447,7 +24294,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24561,7 +24408,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24675,7 +24522,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24789,7 +24636,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24903,7 +24750,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25017,7 +24864,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25131,7 +24978,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25245,7 +25092,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25359,7 +25206,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25473,7 +25320,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25587,7 +25434,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25701,7 +25548,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25815,7 +25662,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25929,7 +25776,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26043,7 +25890,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26157,7 +26004,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26271,7 +26118,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26385,7 +26232,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26499,7 +26346,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26613,7 +26460,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26727,7 +26574,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26841,7 +26688,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26955,7 +26802,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27069,7 +26916,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27082,7 +26929,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -27092,15 +26939,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H231" t="n">
-        <v>3</v>
-      </c>
-      <c r="I231" t="n">
-        <v>0</v>
-      </c>
-      <c r="J231" t="n">
-        <v>3</v>
       </c>
       <c r="K231" t="inlineStr">
         <is>
@@ -27192,7 +27030,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27306,7 +27144,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27420,7 +27258,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27534,7 +27372,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27648,7 +27486,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27661,7 +27499,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -27673,7 +27511,7 @@
         </is>
       </c>
       <c r="H236" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I236" t="n">
         <v>1</v>
@@ -27771,7 +27609,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27784,7 +27622,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F237" t="n">
@@ -27796,7 +27634,7 @@
         </is>
       </c>
       <c r="H237" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I237" t="n">
         <v>1</v>
@@ -27838,10 +27676,10 @@
         </is>
       </c>
       <c r="R237" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S237" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T237" t="n">
         <v>0</v>
@@ -27894,7 +27732,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27907,7 +27745,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F238" t="n">
@@ -27919,7 +27757,7 @@
         </is>
       </c>
       <c r="H238" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I238" t="n">
         <v>1</v>
@@ -28017,7 +27855,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28131,7 +27969,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28245,7 +28083,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28359,7 +28197,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28473,7 +28311,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28587,7 +28425,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28701,7 +28539,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28815,7 +28653,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28929,7 +28767,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29043,7 +28881,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29157,7 +28995,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29271,7 +29109,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29385,7 +29223,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29499,7 +29337,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29613,7 +29451,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29727,7 +29565,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29841,7 +29679,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29955,7 +29793,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30069,7 +29907,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30183,7 +30021,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30297,7 +30135,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30411,7 +30249,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30525,7 +30363,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30639,7 +30477,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30753,7 +30591,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30867,7 +30705,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30981,7 +30819,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31095,7 +30933,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31209,7 +31047,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31323,7 +31161,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31437,7 +31275,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31551,7 +31389,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31665,7 +31503,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31779,7 +31617,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31893,7 +31731,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -32007,7 +31845,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32121,7 +31959,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32235,7 +32073,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32349,7 +32187,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32463,7 +32301,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32577,7 +32415,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32691,7 +32529,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32805,7 +32643,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32818,7 +32656,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -32830,7 +32668,7 @@
         </is>
       </c>
       <c r="H281" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I281" t="n">
         <v>1</v>
@@ -32928,7 +32766,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32941,7 +32779,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -32953,7 +32791,7 @@
         </is>
       </c>
       <c r="H282" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I282" t="n">
         <v>1</v>
@@ -33051,7 +32889,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33064,7 +32902,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F283" t="n">
@@ -33076,7 +32914,7 @@
         </is>
       </c>
       <c r="H283" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I283" t="n">
         <v>1</v>
@@ -33174,7 +33012,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33187,7 +33025,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F284" t="n">
@@ -33199,7 +33037,7 @@
         </is>
       </c>
       <c r="H284" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I284" t="n">
         <v>1</v>
@@ -33297,7 +33135,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33310,7 +33148,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F285" t="n">
@@ -33322,7 +33160,7 @@
         </is>
       </c>
       <c r="H285" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I285" t="n">
         <v>1</v>
@@ -33420,7 +33258,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33433,7 +33271,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F286" t="n">
@@ -33445,7 +33283,7 @@
         </is>
       </c>
       <c r="H286" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I286" t="n">
         <v>1</v>
@@ -33543,7 +33381,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33556,7 +33394,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F287" t="n">
@@ -33568,7 +33406,7 @@
         </is>
       </c>
       <c r="H287" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I287" t="n">
         <v>1</v>
@@ -33666,7 +33504,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33679,7 +33517,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Top 9 | 3 out</t>
         </is>
       </c>
       <c r="F288" t="n">
@@ -33691,7 +33529,7 @@
         </is>
       </c>
       <c r="H288" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I288" t="n">
         <v>1</v>
@@ -33789,7 +33627,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33903,7 +33741,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -34017,7 +33855,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34131,7 +33969,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34245,7 +34083,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34359,7 +34197,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34473,7 +34311,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34587,7 +34425,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34701,7 +34539,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34815,7 +34653,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34929,7 +34767,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -35043,7 +34881,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35157,7 +34995,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35271,7 +35109,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35385,7 +35223,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35499,7 +35337,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35613,7 +35451,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35727,7 +35565,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35841,7 +35679,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35955,7 +35793,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36069,7 +35907,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36183,7 +36021,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36297,7 +36135,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36411,7 +36249,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:52 PM PT</t>
+          <t>2026-07-11 08:51:52 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36525,7 +36363,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36538,7 +36376,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F313" t="n">
@@ -36548,15 +36386,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H313" t="n">
-        <v>3</v>
-      </c>
-      <c r="I313" t="n">
-        <v>0</v>
-      </c>
-      <c r="J313" t="n">
-        <v>3</v>
       </c>
       <c r="K313" t="inlineStr">
         <is>
@@ -36648,7 +36477,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36661,7 +36490,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F314" t="n">
@@ -36671,15 +36500,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H314" t="n">
-        <v>3</v>
-      </c>
-      <c r="I314" t="n">
-        <v>0</v>
-      </c>
-      <c r="J314" t="n">
-        <v>3</v>
       </c>
       <c r="K314" t="inlineStr">
         <is>
@@ -36771,7 +36591,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36885,7 +36705,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36999,7 +36819,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37113,7 +36933,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37227,7 +37047,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37341,7 +37161,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37455,7 +37275,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37569,7 +37389,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37683,7 +37503,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37797,7 +37617,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37911,7 +37731,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -38025,7 +37845,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -38139,7 +37959,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38253,7 +38073,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38367,7 +38187,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38481,7 +38301,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38595,7 +38415,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38709,7 +38529,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38823,7 +38643,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38937,7 +38757,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -39051,7 +38871,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:54 PM PT</t>
+          <t>2026-07-11 08:51:54 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -39064,7 +38884,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F335" t="n">
@@ -39074,15 +38894,6 @@
         <is>
           <t>Top</t>
         </is>
-      </c>
-      <c r="H335" t="n">
-        <v>3</v>
-      </c>
-      <c r="I335" t="n">
-        <v>0</v>
-      </c>
-      <c r="J335" t="n">
-        <v>3</v>
       </c>
       <c r="K335" t="inlineStr">
         <is>
@@ -39174,7 +38985,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -39288,7 +39099,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 08:49:53 PM PT</t>
+          <t>2026-07-11 08:51:53 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:53:56 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -487,7 +487,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -828,17 +828,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -930,7 +930,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -2775,17 +2775,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -3240,17 +3240,17 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -5415,17 +5415,17 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -5517,7 +5517,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6543,7 +6543,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6670,7 +6670,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -6678,17 +6678,17 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H54" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7350,7 +7350,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8376,7 +8376,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8739,17 +8739,17 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -8841,7 +8841,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9297,7 +9297,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9981,7 +9981,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10209,7 +10209,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10437,7 +10437,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10665,7 +10665,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11134,7 +11134,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11142,17 +11142,17 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H93" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J93" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -11244,7 +11244,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11358,7 +11358,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11700,7 +11700,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11827,7 +11827,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11835,17 +11835,17 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H99" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J99" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -11937,7 +11937,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12051,7 +12051,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12165,7 +12165,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12279,7 +12279,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12507,7 +12507,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12621,7 +12621,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12735,7 +12735,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12849,7 +12849,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12963,7 +12963,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13191,7 +13191,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13305,7 +13305,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13419,7 +13419,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13533,7 +13533,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13647,7 +13647,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13761,7 +13761,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13875,7 +13875,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14103,7 +14103,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14217,7 +14217,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14445,7 +14445,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14559,7 +14559,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14673,7 +14673,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15015,7 +15015,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15129,7 +15129,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15243,7 +15243,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15357,7 +15357,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15471,7 +15471,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -15492,17 +15492,17 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H131" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -15594,7 +15594,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15708,7 +15708,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15822,7 +15822,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15936,7 +15936,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16050,7 +16050,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16164,7 +16164,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16278,7 +16278,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16392,7 +16392,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16506,7 +16506,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16620,7 +16620,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16734,7 +16734,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16962,7 +16962,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17076,7 +17076,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17190,7 +17190,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17304,7 +17304,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17418,7 +17418,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17532,7 +17532,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17646,7 +17646,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17760,7 +17760,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17874,7 +17874,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17988,7 +17988,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18102,7 +18102,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18216,7 +18216,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18330,7 +18330,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18444,7 +18444,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18558,7 +18558,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18786,7 +18786,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18900,7 +18900,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19128,7 +19128,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19242,7 +19242,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19356,7 +19356,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19470,7 +19470,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19584,7 +19584,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19698,7 +19698,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19812,7 +19812,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19926,7 +19926,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20040,7 +20040,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20154,7 +20154,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20167,7 +20167,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20175,17 +20175,17 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H172" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I172" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J172" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20277,7 +20277,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20290,7 +20290,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -20298,17 +20298,17 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H173" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I173" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J173" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K173" t="inlineStr">
         <is>
@@ -20400,7 +20400,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20514,7 +20514,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20628,7 +20628,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20742,7 +20742,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20856,7 +20856,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20970,7 +20970,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21084,7 +21084,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21198,7 +21198,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21312,7 +21312,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21540,7 +21540,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21768,7 +21768,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21882,7 +21882,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21996,7 +21996,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22110,7 +22110,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22224,7 +22224,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22338,7 +22338,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22452,7 +22452,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22566,7 +22566,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22680,7 +22680,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22693,7 +22693,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -22701,17 +22701,17 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H194" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I194" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J194" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K194" t="inlineStr">
         <is>
@@ -22803,7 +22803,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22816,7 +22816,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -22824,17 +22824,17 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H195" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I195" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J195" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K195" t="inlineStr">
         <is>
@@ -22926,7 +22926,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23040,7 +23040,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23154,7 +23154,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23268,7 +23268,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23382,7 +23382,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23496,7 +23496,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23610,7 +23610,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23724,7 +23724,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23838,7 +23838,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23952,7 +23952,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24066,7 +24066,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24180,7 +24180,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24294,7 +24294,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24408,7 +24408,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24522,7 +24522,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24636,7 +24636,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24750,7 +24750,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24864,7 +24864,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24978,7 +24978,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25092,7 +25092,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25320,7 +25320,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25434,7 +25434,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25548,7 +25548,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25662,7 +25662,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25776,7 +25776,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25890,7 +25890,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26004,7 +26004,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26118,7 +26118,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26232,7 +26232,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26346,7 +26346,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26460,7 +26460,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26574,7 +26574,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26688,7 +26688,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26802,7 +26802,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26916,7 +26916,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27030,7 +27030,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27144,7 +27144,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27258,7 +27258,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27372,7 +27372,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27486,7 +27486,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27499,7 +27499,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -27507,17 +27507,17 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H236" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I236" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J236" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K236" t="inlineStr">
         <is>
@@ -27609,7 +27609,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27622,7 +27622,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F237" t="n">
@@ -27630,17 +27630,17 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H237" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I237" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J237" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K237" t="inlineStr">
         <is>
@@ -27667,7 +27667,7 @@
       </c>
       <c r="P237" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="Q237" t="inlineStr">
@@ -27732,7 +27732,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27745,7 +27745,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F238" t="n">
@@ -27753,17 +27753,17 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H238" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I238" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J238" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K238" t="inlineStr">
         <is>
@@ -27855,7 +27855,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27969,7 +27969,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28311,7 +28311,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28539,7 +28539,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28653,7 +28653,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28767,7 +28767,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28995,7 +28995,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29109,7 +29109,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29223,7 +29223,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29565,7 +29565,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29679,7 +29679,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29793,7 +29793,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29907,7 +29907,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30021,7 +30021,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30135,7 +30135,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30363,7 +30363,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30591,7 +30591,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30705,7 +30705,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30819,7 +30819,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31047,7 +31047,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31161,7 +31161,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31275,7 +31275,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31389,7 +31389,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31503,7 +31503,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31617,7 +31617,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31731,7 +31731,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31845,7 +31845,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31959,7 +31959,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32073,7 +32073,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32187,7 +32187,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32301,7 +32301,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32415,7 +32415,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32529,7 +32529,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32643,7 +32643,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32656,7 +32656,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -32664,17 +32664,17 @@
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H281" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I281" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J281" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K281" t="inlineStr">
         <is>
@@ -32766,7 +32766,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32779,7 +32779,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -32787,17 +32787,17 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H282" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I282" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J282" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K282" t="inlineStr">
         <is>
@@ -32889,7 +32889,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32902,7 +32902,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F283" t="n">
@@ -32910,17 +32910,17 @@
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H283" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I283" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J283" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K283" t="inlineStr">
         <is>
@@ -33012,7 +33012,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33025,7 +33025,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F284" t="n">
@@ -33033,17 +33033,17 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H284" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I284" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J284" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K284" t="inlineStr">
         <is>
@@ -33135,7 +33135,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33148,7 +33148,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F285" t="n">
@@ -33156,17 +33156,17 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H285" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I285" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J285" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K285" t="inlineStr">
         <is>
@@ -33258,7 +33258,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33271,7 +33271,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F286" t="n">
@@ -33279,17 +33279,17 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H286" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I286" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J286" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K286" t="inlineStr">
         <is>
@@ -33381,7 +33381,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33394,7 +33394,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F287" t="n">
@@ -33402,17 +33402,17 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H287" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I287" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J287" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K287" t="inlineStr">
         <is>
@@ -33504,7 +33504,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33517,7 +33517,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Top 9 | 3 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F288" t="n">
@@ -33525,17 +33525,17 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H288" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I288" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J288" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K288" t="inlineStr">
         <is>
@@ -33627,7 +33627,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33741,7 +33741,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33855,7 +33855,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33969,7 +33969,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34083,7 +34083,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34197,7 +34197,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34311,7 +34311,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34539,7 +34539,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34653,7 +34653,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34767,7 +34767,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34881,7 +34881,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34995,7 +34995,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35109,7 +35109,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35223,7 +35223,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35337,7 +35337,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35451,7 +35451,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35565,7 +35565,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35679,7 +35679,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35793,7 +35793,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35907,7 +35907,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36021,7 +36021,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36135,7 +36135,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:52 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36249,7 +36249,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:52 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36363,7 +36363,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36477,7 +36477,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36591,7 +36591,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36705,7 +36705,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36819,7 +36819,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36933,7 +36933,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37047,7 +37047,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37161,7 +37161,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37275,7 +37275,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37389,7 +37389,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37503,7 +37503,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37617,7 +37617,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37731,7 +37731,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37845,7 +37845,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37959,7 +37959,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38073,7 +38073,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38187,7 +38187,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38301,7 +38301,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38415,7 +38415,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38529,7 +38529,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38643,7 +38643,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38757,7 +38757,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38871,7 +38871,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:54 PM PT</t>
+          <t>2026-07-11 08:53:54 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38985,7 +38985,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -39099,7 +39099,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 08:51:53 PM PT</t>
+          <t>2026-07-11 08:53:53 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:55:55 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -930,7 +930,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -2779,7 +2779,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -3244,7 +3244,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5407,7 +5407,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
@@ -5517,7 +5517,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6543,7 +6543,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6670,7 +6670,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -6682,7 +6682,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7350,7 +7350,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8376,7 +8376,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8743,7 +8743,7 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I72" t="n">
         <v>0</v>
@@ -8841,7 +8841,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9297,7 +9297,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9981,7 +9981,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10209,7 +10209,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10437,7 +10437,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10665,7 +10665,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11134,7 +11134,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11146,7 +11146,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I93" t="n">
         <v>0</v>
@@ -11244,7 +11244,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11358,7 +11358,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11700,7 +11700,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11827,7 +11827,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11839,7 +11839,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -11937,7 +11937,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12051,7 +12051,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12165,7 +12165,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12279,7 +12279,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12507,7 +12507,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12621,7 +12621,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12735,7 +12735,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12849,7 +12849,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12963,7 +12963,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13191,7 +13191,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13305,7 +13305,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13419,7 +13419,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13533,7 +13533,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13647,7 +13647,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13761,7 +13761,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13875,7 +13875,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14103,7 +14103,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14217,7 +14217,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14445,7 +14445,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14559,7 +14559,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14673,7 +14673,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15015,7 +15015,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15129,7 +15129,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15243,7 +15243,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15357,7 +15357,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15471,7 +15471,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -15496,7 +15496,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I131" t="n">
         <v>0</v>
@@ -15594,7 +15594,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15708,7 +15708,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15822,7 +15822,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15936,7 +15936,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16050,7 +16050,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16164,7 +16164,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16278,7 +16278,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16392,7 +16392,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16506,7 +16506,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16620,7 +16620,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16734,7 +16734,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16962,7 +16962,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17076,7 +17076,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17190,7 +17190,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17304,7 +17304,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17418,7 +17418,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17532,7 +17532,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17646,7 +17646,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17760,7 +17760,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17874,7 +17874,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17988,7 +17988,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18102,7 +18102,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18216,7 +18216,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18330,7 +18330,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18444,7 +18444,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18558,7 +18558,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18786,7 +18786,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18900,7 +18900,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19128,7 +19128,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19242,7 +19242,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19356,7 +19356,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19470,7 +19470,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19584,7 +19584,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19698,7 +19698,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19812,7 +19812,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19926,7 +19926,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20040,7 +20040,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20154,7 +20154,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20167,7 +20167,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20179,7 +20179,7 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I172" t="n">
         <v>0</v>
@@ -20277,7 +20277,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20290,7 +20290,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -20302,7 +20302,7 @@
         </is>
       </c>
       <c r="H173" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I173" t="n">
         <v>0</v>
@@ -20400,7 +20400,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20514,7 +20514,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20628,7 +20628,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20742,7 +20742,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20856,7 +20856,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20970,7 +20970,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21084,7 +21084,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21198,7 +21198,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21312,7 +21312,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21540,7 +21540,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21768,7 +21768,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21882,7 +21882,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21996,7 +21996,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22110,7 +22110,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22224,7 +22224,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22338,7 +22338,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22452,7 +22452,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22566,7 +22566,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22680,7 +22680,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22693,7 +22693,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -22705,7 +22705,7 @@
         </is>
       </c>
       <c r="H194" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I194" t="n">
         <v>0</v>
@@ -22803,7 +22803,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22816,7 +22816,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -22828,7 +22828,7 @@
         </is>
       </c>
       <c r="H195" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I195" t="n">
         <v>0</v>
@@ -22926,7 +22926,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23040,7 +23040,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23154,7 +23154,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23268,7 +23268,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23382,7 +23382,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23496,7 +23496,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23610,7 +23610,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23724,7 +23724,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23838,7 +23838,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23952,7 +23952,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24066,7 +24066,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24180,7 +24180,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24294,7 +24294,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24408,7 +24408,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24522,7 +24522,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24636,7 +24636,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24750,7 +24750,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24864,7 +24864,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24978,7 +24978,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25092,7 +25092,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25320,7 +25320,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25434,7 +25434,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25548,7 +25548,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25662,7 +25662,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25776,7 +25776,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25890,7 +25890,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26004,7 +26004,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26118,7 +26118,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26232,7 +26232,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26346,7 +26346,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26460,7 +26460,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26574,7 +26574,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26688,7 +26688,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26802,7 +26802,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26916,7 +26916,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27030,7 +27030,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27144,7 +27144,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27258,7 +27258,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27372,7 +27372,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27486,7 +27486,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27499,7 +27499,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -27511,7 +27511,7 @@
         </is>
       </c>
       <c r="H236" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
@@ -27609,7 +27609,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27622,7 +27622,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F237" t="n">
@@ -27634,7 +27634,7 @@
         </is>
       </c>
       <c r="H237" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I237" t="n">
         <v>0</v>
@@ -27732,7 +27732,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27745,7 +27745,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F238" t="n">
@@ -27757,7 +27757,7 @@
         </is>
       </c>
       <c r="H238" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I238" t="n">
         <v>0</v>
@@ -27855,7 +27855,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27969,7 +27969,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28311,7 +28311,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28539,7 +28539,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28653,7 +28653,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28767,7 +28767,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28995,7 +28995,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29109,7 +29109,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29223,7 +29223,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29565,7 +29565,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29679,7 +29679,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29793,7 +29793,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29907,7 +29907,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30021,7 +30021,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30135,7 +30135,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30363,7 +30363,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30591,7 +30591,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30705,7 +30705,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30819,7 +30819,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31047,7 +31047,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31161,7 +31161,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31275,7 +31275,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31389,7 +31389,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31503,7 +31503,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31617,7 +31617,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31731,7 +31731,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31845,7 +31845,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31959,7 +31959,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32073,7 +32073,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32187,7 +32187,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32301,7 +32301,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32415,7 +32415,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32529,7 +32529,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32643,7 +32643,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32656,7 +32656,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -32668,7 +32668,7 @@
         </is>
       </c>
       <c r="H281" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I281" t="n">
         <v>0</v>
@@ -32766,7 +32766,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32779,7 +32779,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -32791,7 +32791,7 @@
         </is>
       </c>
       <c r="H282" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I282" t="n">
         <v>0</v>
@@ -32889,7 +32889,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32902,7 +32902,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F283" t="n">
@@ -32914,7 +32914,7 @@
         </is>
       </c>
       <c r="H283" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I283" t="n">
         <v>0</v>
@@ -32956,10 +32956,10 @@
         </is>
       </c>
       <c r="R283" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S283" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T283" t="n">
         <v>0</v>
@@ -33012,7 +33012,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33025,7 +33025,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F284" t="n">
@@ -33037,7 +33037,7 @@
         </is>
       </c>
       <c r="H284" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I284" t="n">
         <v>0</v>
@@ -33079,10 +33079,10 @@
         </is>
       </c>
       <c r="R284" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S284" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T284" t="n">
         <v>0</v>
@@ -33135,7 +33135,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33148,7 +33148,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F285" t="n">
@@ -33160,7 +33160,7 @@
         </is>
       </c>
       <c r="H285" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I285" t="n">
         <v>0</v>
@@ -33258,7 +33258,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33271,7 +33271,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F286" t="n">
@@ -33283,7 +33283,7 @@
         </is>
       </c>
       <c r="H286" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I286" t="n">
         <v>0</v>
@@ -33381,7 +33381,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33394,7 +33394,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F287" t="n">
@@ -33406,7 +33406,7 @@
         </is>
       </c>
       <c r="H287" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I287" t="n">
         <v>0</v>
@@ -33504,7 +33504,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33517,7 +33517,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 2 out</t>
         </is>
       </c>
       <c r="F288" t="n">
@@ -33529,7 +33529,7 @@
         </is>
       </c>
       <c r="H288" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I288" t="n">
         <v>0</v>
@@ -33627,7 +33627,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33741,7 +33741,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33855,7 +33855,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33969,7 +33969,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34083,7 +34083,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34197,7 +34197,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34311,7 +34311,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34539,7 +34539,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34653,7 +34653,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34767,7 +34767,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34881,7 +34881,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34995,7 +34995,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35109,7 +35109,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35223,7 +35223,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35337,7 +35337,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35451,7 +35451,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35565,7 +35565,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35679,7 +35679,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35793,7 +35793,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35907,7 +35907,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36021,7 +36021,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36135,7 +36135,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:52 PM PT</t>
+          <t>2026-07-11 08:55:52 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36249,7 +36249,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36363,7 +36363,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36477,7 +36477,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36591,7 +36591,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36705,7 +36705,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36819,7 +36819,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36933,7 +36933,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37047,7 +37047,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37161,7 +37161,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37275,7 +37275,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37389,7 +37389,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37503,7 +37503,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37617,7 +37617,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37731,7 +37731,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37845,7 +37845,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37959,7 +37959,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38073,7 +38073,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38187,7 +38187,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38301,7 +38301,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38415,7 +38415,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38529,7 +38529,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38643,7 +38643,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38757,7 +38757,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38871,7 +38871,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:54 PM PT</t>
+          <t>2026-07-11 08:55:54 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38985,7 +38985,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -39099,7 +39099,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 08:53:53 PM PT</t>
+          <t>2026-07-11 08:55:53 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:56:06 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -930,7 +930,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5631,7 +5631,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6429,7 +6429,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6543,7 +6543,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7350,7 +7350,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8376,7 +8376,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8604,7 +8604,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9183,7 +9183,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9297,7 +9297,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9411,7 +9411,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9525,7 +9525,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9867,7 +9867,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9981,7 +9981,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10209,7 +10209,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10323,7 +10323,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10437,7 +10437,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10665,7 +10665,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10893,7 +10893,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11007,7 +11007,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11244,7 +11244,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11358,7 +11358,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11700,7 +11700,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11937,7 +11937,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12051,7 +12051,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12165,7 +12165,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12279,7 +12279,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12507,7 +12507,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12621,7 +12621,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12735,7 +12735,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12849,7 +12849,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12963,7 +12963,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13191,7 +13191,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13305,7 +13305,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13419,7 +13419,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13533,7 +13533,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13647,7 +13647,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13761,7 +13761,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13875,7 +13875,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14103,7 +14103,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14217,7 +14217,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14445,7 +14445,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14559,7 +14559,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14673,7 +14673,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15015,7 +15015,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15129,7 +15129,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15243,7 +15243,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15357,7 +15357,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15471,7 +15471,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15594,7 +15594,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15708,7 +15708,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15822,7 +15822,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15936,7 +15936,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16050,7 +16050,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16164,7 +16164,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16278,7 +16278,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16392,7 +16392,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16506,7 +16506,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16620,7 +16620,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16734,7 +16734,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16848,7 +16848,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16962,7 +16962,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17076,7 +17076,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17190,7 +17190,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17304,7 +17304,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17418,7 +17418,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17532,7 +17532,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17646,7 +17646,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17760,7 +17760,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17874,7 +17874,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17988,7 +17988,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18102,7 +18102,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18216,7 +18216,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18330,7 +18330,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18444,7 +18444,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18558,7 +18558,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18786,7 +18786,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18900,7 +18900,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19128,7 +19128,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19242,7 +19242,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19356,7 +19356,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19470,7 +19470,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19584,7 +19584,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19698,7 +19698,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19812,7 +19812,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19926,7 +19926,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20040,7 +20040,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20154,7 +20154,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20277,7 +20277,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20400,7 +20400,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20514,7 +20514,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20628,7 +20628,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20742,7 +20742,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20856,7 +20856,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20970,7 +20970,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21084,7 +21084,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21198,7 +21198,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21312,7 +21312,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21426,7 +21426,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21540,7 +21540,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21768,7 +21768,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21882,7 +21882,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21996,7 +21996,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22110,7 +22110,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22224,7 +22224,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22338,7 +22338,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22452,7 +22452,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22566,7 +22566,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22680,7 +22680,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22803,7 +22803,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22926,7 +22926,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23040,7 +23040,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23154,7 +23154,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23268,7 +23268,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23382,7 +23382,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23496,7 +23496,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23610,7 +23610,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23724,7 +23724,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23838,7 +23838,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23952,7 +23952,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24066,7 +24066,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24180,7 +24180,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24294,7 +24294,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24408,7 +24408,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24522,7 +24522,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24636,7 +24636,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24750,7 +24750,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24864,7 +24864,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24978,7 +24978,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25092,7 +25092,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25206,7 +25206,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25320,7 +25320,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25434,7 +25434,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25548,7 +25548,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25662,7 +25662,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25776,7 +25776,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25890,7 +25890,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26004,7 +26004,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26118,7 +26118,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26232,7 +26232,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26346,7 +26346,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26460,7 +26460,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26574,7 +26574,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26688,7 +26688,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26802,7 +26802,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26916,7 +26916,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27030,7 +27030,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27144,7 +27144,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27258,7 +27258,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27372,7 +27372,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27486,7 +27486,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27609,7 +27609,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27732,7 +27732,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27855,7 +27855,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27969,7 +27969,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28311,7 +28311,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28539,7 +28539,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28653,7 +28653,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28767,7 +28767,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28995,7 +28995,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29109,7 +29109,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29223,7 +29223,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29565,7 +29565,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29679,7 +29679,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29793,7 +29793,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29907,7 +29907,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30021,7 +30021,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30135,7 +30135,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30363,7 +30363,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30591,7 +30591,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30705,7 +30705,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30819,7 +30819,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31047,7 +31047,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31161,7 +31161,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31275,7 +31275,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31389,7 +31389,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31503,7 +31503,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31617,7 +31617,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31731,7 +31731,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31845,7 +31845,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31959,7 +31959,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32073,7 +32073,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32187,7 +32187,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32301,7 +32301,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32415,7 +32415,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32529,7 +32529,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32643,7 +32643,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32766,7 +32766,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32889,7 +32889,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33012,7 +33012,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33135,7 +33135,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33258,7 +33258,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33381,7 +33381,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33504,7 +33504,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33627,7 +33627,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33741,7 +33741,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33855,7 +33855,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33969,7 +33969,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34083,7 +34083,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34197,7 +34197,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34311,7 +34311,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34425,7 +34425,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34539,7 +34539,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34653,7 +34653,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34767,7 +34767,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34881,7 +34881,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34995,7 +34995,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35109,7 +35109,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35223,7 +35223,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35337,7 +35337,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35451,7 +35451,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35565,7 +35565,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35679,7 +35679,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35793,7 +35793,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35907,7 +35907,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36021,7 +36021,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36135,7 +36135,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:52 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36249,7 +36249,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36363,7 +36363,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36477,7 +36477,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36591,7 +36591,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36705,7 +36705,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36819,7 +36819,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36933,7 +36933,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37047,7 +37047,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37161,7 +37161,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37275,7 +37275,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37389,7 +37389,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37503,7 +37503,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37617,7 +37617,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37731,7 +37731,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37845,7 +37845,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37959,7 +37959,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38073,7 +38073,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38187,7 +38187,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38301,7 +38301,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38415,7 +38415,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38529,7 +38529,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38643,7 +38643,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38757,7 +38757,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38871,7 +38871,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:54 PM PT</t>
+          <t>2026-07-11 08:56:04 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38985,7 +38985,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -39099,7 +39099,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 08:55:53 PM PT</t>
+          <t>2026-07-11 08:56:03 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 08:58:05 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -487,7 +487,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -830,15 +830,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -930,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1044,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1158,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1272,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1386,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1500,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1614,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2767,7 +2758,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -2777,15 +2768,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H20" t="n">
-        <v>2</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2877,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2991,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3105,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3219,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3232,7 +3214,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -3242,15 +3224,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H24" t="n">
-        <v>2</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -3342,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3456,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3570,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3684,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3798,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3912,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4026,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4140,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4254,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4368,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4482,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4596,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4710,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4824,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4938,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5052,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5166,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5280,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5394,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5407,7 +5380,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -5417,15 +5390,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H43" t="n">
-        <v>2</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -5517,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5631,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5745,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5859,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5973,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6087,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6201,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6315,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6429,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6543,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6657,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6670,7 +6634,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -6680,15 +6644,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H54" t="n">
-        <v>2</v>
-      </c>
-      <c r="I54" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" t="n">
-        <v>0</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
@@ -6780,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7236,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7350,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7464,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7578,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7692,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7806,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7920,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8034,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8148,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8262,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8376,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8490,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8604,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8718,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8731,7 +8686,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8741,15 +8696,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H72" t="n">
-        <v>2</v>
-      </c>
-      <c r="I72" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" t="n">
-        <v>0</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -8841,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8955,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9069,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9183,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9297,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9411,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9525,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9639,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9753,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9867,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9981,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10095,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10209,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10323,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10437,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10551,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10665,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10779,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10893,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11007,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11121,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11134,7 +11080,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11144,15 +11090,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H93" t="n">
-        <v>2</v>
-      </c>
-      <c r="I93" t="n">
-        <v>0</v>
-      </c>
-      <c r="J93" t="n">
-        <v>0</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -11244,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11358,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11472,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11586,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11700,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11814,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11827,7 +11764,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11837,15 +11774,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H99" t="n">
-        <v>2</v>
-      </c>
-      <c r="I99" t="n">
-        <v>0</v>
-      </c>
-      <c r="J99" t="n">
-        <v>0</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -11937,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12051,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12165,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12279,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12393,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12507,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12621,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12735,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12849,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12963,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13077,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13191,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13305,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13419,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13533,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13647,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13761,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13875,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13989,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14103,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14217,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14331,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14445,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14559,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14673,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14787,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14901,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15015,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15129,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15243,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15357,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15471,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15484,7 +15412,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -15494,15 +15422,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H131" t="n">
-        <v>2</v>
-      </c>
-      <c r="I131" t="n">
-        <v>0</v>
-      </c>
-      <c r="J131" t="n">
-        <v>0</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -15594,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15708,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15822,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15936,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16050,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16164,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16278,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16392,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16506,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16620,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16734,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16848,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16962,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17076,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17190,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17304,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17418,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17532,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17646,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17760,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17874,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17988,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18102,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18216,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18330,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18444,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18558,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18672,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18786,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18900,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19014,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19128,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19242,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19356,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19470,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19584,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19698,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19812,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19926,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20040,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20154,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20167,7 +20086,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20177,15 +20096,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H172" t="n">
-        <v>2</v>
-      </c>
-      <c r="I172" t="n">
-        <v>0</v>
-      </c>
-      <c r="J172" t="n">
-        <v>0</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20277,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20290,7 +20200,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -20300,15 +20210,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H173" t="n">
-        <v>2</v>
-      </c>
-      <c r="I173" t="n">
-        <v>0</v>
-      </c>
-      <c r="J173" t="n">
-        <v>0</v>
       </c>
       <c r="K173" t="inlineStr">
         <is>
@@ -20400,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20514,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20628,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20742,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20856,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20970,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21084,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21198,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21312,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21426,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21540,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21654,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21768,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21882,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21996,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22110,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22224,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22338,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22452,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22566,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22680,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22693,7 +22594,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -22703,15 +22604,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H194" t="n">
-        <v>2</v>
-      </c>
-      <c r="I194" t="n">
-        <v>0</v>
-      </c>
-      <c r="J194" t="n">
-        <v>0</v>
       </c>
       <c r="K194" t="inlineStr">
         <is>
@@ -22803,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22816,7 +22708,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -22826,15 +22718,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H195" t="n">
-        <v>2</v>
-      </c>
-      <c r="I195" t="n">
-        <v>0</v>
-      </c>
-      <c r="J195" t="n">
-        <v>0</v>
       </c>
       <c r="K195" t="inlineStr">
         <is>
@@ -22926,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23040,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23154,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23268,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23382,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23496,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23610,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23724,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23838,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23952,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24066,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24180,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24294,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24408,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24522,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24636,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24750,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24864,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24978,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25092,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25206,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25320,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25434,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25548,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25662,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25776,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25890,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26004,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26118,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26232,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26346,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26460,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26574,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26688,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26802,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26916,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27030,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27144,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27258,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27372,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27486,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27499,7 +27382,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -27509,15 +27392,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H236" t="n">
-        <v>2</v>
-      </c>
-      <c r="I236" t="n">
-        <v>0</v>
-      </c>
-      <c r="J236" t="n">
-        <v>0</v>
       </c>
       <c r="K236" t="inlineStr">
         <is>
@@ -27609,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27622,7 +27496,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F237" t="n">
@@ -27632,15 +27506,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H237" t="n">
-        <v>2</v>
-      </c>
-      <c r="I237" t="n">
-        <v>0</v>
-      </c>
-      <c r="J237" t="n">
-        <v>0</v>
       </c>
       <c r="K237" t="inlineStr">
         <is>
@@ -27732,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27745,7 +27610,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F238" t="n">
@@ -27755,15 +27620,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H238" t="n">
-        <v>2</v>
-      </c>
-      <c r="I238" t="n">
-        <v>0</v>
-      </c>
-      <c r="J238" t="n">
-        <v>0</v>
       </c>
       <c r="K238" t="inlineStr">
         <is>
@@ -27855,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27969,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28083,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28197,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28311,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28425,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28539,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28653,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28767,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28881,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28995,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29109,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29223,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29337,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29451,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29565,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29679,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29793,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29907,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30021,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30135,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30249,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30363,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30477,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30591,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30705,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30819,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30933,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31047,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31161,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31275,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31389,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31503,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31617,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31731,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31845,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31959,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32073,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32187,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32301,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32415,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32529,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32643,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32656,7 +32512,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -32666,15 +32522,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H281" t="n">
-        <v>2</v>
-      </c>
-      <c r="I281" t="n">
-        <v>0</v>
-      </c>
-      <c r="J281" t="n">
-        <v>0</v>
       </c>
       <c r="K281" t="inlineStr">
         <is>
@@ -32766,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32779,7 +32626,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -32789,15 +32636,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H282" t="n">
-        <v>2</v>
-      </c>
-      <c r="I282" t="n">
-        <v>0</v>
-      </c>
-      <c r="J282" t="n">
-        <v>0</v>
       </c>
       <c r="K282" t="inlineStr">
         <is>
@@ -32889,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32902,7 +32740,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F283" t="n">
@@ -32912,15 +32750,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H283" t="n">
-        <v>2</v>
-      </c>
-      <c r="I283" t="n">
-        <v>0</v>
-      </c>
-      <c r="J283" t="n">
-        <v>0</v>
       </c>
       <c r="K283" t="inlineStr">
         <is>
@@ -33012,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33025,7 +32854,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F284" t="n">
@@ -33035,15 +32864,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H284" t="n">
-        <v>2</v>
-      </c>
-      <c r="I284" t="n">
-        <v>0</v>
-      </c>
-      <c r="J284" t="n">
-        <v>0</v>
       </c>
       <c r="K284" t="inlineStr">
         <is>
@@ -33135,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33148,7 +32968,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F285" t="n">
@@ -33158,15 +32978,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H285" t="n">
-        <v>2</v>
-      </c>
-      <c r="I285" t="n">
-        <v>0</v>
-      </c>
-      <c r="J285" t="n">
-        <v>0</v>
       </c>
       <c r="K285" t="inlineStr">
         <is>
@@ -33202,10 +33013,10 @@
         </is>
       </c>
       <c r="R285" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S285" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T285" t="n">
         <v>0</v>
@@ -33258,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33271,7 +33082,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F286" t="n">
@@ -33281,15 +33092,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H286" t="n">
-        <v>2</v>
-      </c>
-      <c r="I286" t="n">
-        <v>0</v>
-      </c>
-      <c r="J286" t="n">
-        <v>0</v>
       </c>
       <c r="K286" t="inlineStr">
         <is>
@@ -33381,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33394,7 +33196,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F287" t="n">
@@ -33404,15 +33206,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H287" t="n">
-        <v>2</v>
-      </c>
-      <c r="I287" t="n">
-        <v>0</v>
-      </c>
-      <c r="J287" t="n">
-        <v>0</v>
       </c>
       <c r="K287" t="inlineStr">
         <is>
@@ -33504,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33517,7 +33310,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Bottom 9 | 2 out</t>
+          <t>Game Over</t>
         </is>
       </c>
       <c r="F288" t="n">
@@ -33527,15 +33320,6 @@
         <is>
           <t>Bottom</t>
         </is>
-      </c>
-      <c r="H288" t="n">
-        <v>2</v>
-      </c>
-      <c r="I288" t="n">
-        <v>0</v>
-      </c>
-      <c r="J288" t="n">
-        <v>0</v>
       </c>
       <c r="K288" t="inlineStr">
         <is>
@@ -33627,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33741,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33855,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33969,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34083,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34197,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34311,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34425,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34539,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34653,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34767,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34881,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34995,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35109,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35223,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35337,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35451,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35565,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35679,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35793,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35907,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36021,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36135,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:02 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36249,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36363,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36477,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36591,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36705,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36819,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36933,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37047,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37161,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37275,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37389,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37503,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37617,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37731,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37845,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37959,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -38073,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -38187,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38301,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38415,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38529,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38643,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38757,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38871,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:04 PM PT</t>
+          <t>2026-07-11 08:58:04 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38985,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -39099,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 08:56:03 PM PT</t>
+          <t>2026-07-11 08:58:03 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 09:00:07 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:02 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:04 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:04 PM PT</t>
+          <t>2026-07-11 09:00:05 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 08:58:03 PM PT</t>
+          <t>2026-07-11 09:00:03 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 09:02:06 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:04 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:05 PM PT</t>
+          <t>2026-07-11 09:02:04 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 09:00:03 PM PT</t>
+          <t>2026-07-11 09:02:03 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:26:57 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6520,7 +6520,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8002,7 +8002,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8686,7 +8686,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9256,7 +9256,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11080,7 +11080,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11764,7 +11764,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12334,7 +12334,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13132,7 +13132,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13816,7 +13816,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -13930,7 +13930,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15412,7 +15412,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17464,7 +17464,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18604,7 +18604,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18718,7 +18718,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20086,7 +20086,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20200,7 +20200,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22252,7 +22252,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22594,7 +22594,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22708,7 +22708,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26812,7 +26812,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27382,7 +27382,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27496,7 +27496,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27610,7 +27610,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32512,7 +32512,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32626,7 +32626,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32740,7 +32740,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32854,7 +32854,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -32968,7 +32968,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33082,7 +33082,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33196,7 +33196,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33310,7 +33310,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36160,7 +36160,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36274,7 +36274,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:04 PM PT</t>
+          <t>2026-07-11 10:26:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38668,7 +38668,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 09:02:03 PM PT</t>
+          <t>2026-07-11 10:26:54 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:28:56 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:53 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:55 PM PT</t>
+          <t>2026-07-11 10:28:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 10:26:54 PM PT</t>
+          <t>2026-07-11 10:28:54 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:30:56 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:53 PM PT</t>
+          <t>2026-07-11 10:30:53 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:55 PM PT</t>
+          <t>2026-07-11 10:30:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 10:28:54 PM PT</t>
+          <t>2026-07-11 10:30:54 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:32:56 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:53 PM PT</t>
+          <t>2026-07-11 10:32:53 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:55 PM PT</t>
+          <t>2026-07-11 10:32:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 10:30:54 PM PT</t>
+          <t>2026-07-11 10:32:54 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:34:56 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:53 PM PT</t>
+          <t>2026-07-11 10:34:53 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:55 PM PT</t>
+          <t>2026-07-11 10:34:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 10:32:54 PM PT</t>
+          <t>2026-07-11 10:34:54 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:36:57 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:56 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:53 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:55 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 10:34:54 PM PT</t>
+          <t>2026-07-11 10:36:55 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:38:57 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:56 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:54 PM PT</t>
+          <t>2026-07-11 10:38:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 10:36:55 PM PT</t>
+          <t>2026-07-11 10:38:55 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:40:57 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:56 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:54 PM PT</t>
+          <t>2026-07-11 10:40:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 10:38:55 PM PT</t>
+          <t>2026-07-11 10:40:55 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:42:57 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:56 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:54 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 10:40:55 PM PT</t>
+          <t>2026-07-11 10:42:55 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:44:57 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5481,7 +5481,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5709,7 +5709,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5823,7 +5823,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5937,7 +5937,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6051,7 +6051,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6393,7 +6393,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6849,7 +6849,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7419,7 +7419,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7647,7 +7647,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8103,7 +8103,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8217,7 +8217,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8673,7 +8673,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8787,7 +8787,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9015,7 +9015,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9585,7 +9585,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9813,7 +9813,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9927,7 +9927,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10041,7 +10041,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10155,7 +10155,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10383,7 +10383,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10497,7 +10497,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10725,7 +10725,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11181,7 +11181,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11637,7 +11637,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11979,7 +11979,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12093,7 +12093,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12321,7 +12321,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12777,7 +12777,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13005,7 +13005,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13233,7 +13233,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13575,7 +13575,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13689,7 +13689,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13803,7 +13803,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14145,7 +14145,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14373,7 +14373,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14487,7 +14487,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14715,7 +14715,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14943,7 +14943,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15057,7 +15057,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15399,7 +15399,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15513,7 +15513,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15741,7 +15741,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16197,7 +16197,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16311,7 +16311,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16425,7 +16425,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16539,7 +16539,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16767,7 +16767,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -16995,7 +16995,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17223,7 +17223,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17337,7 +17337,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17451,7 +17451,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17565,7 +17565,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17679,7 +17679,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18249,7 +18249,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18363,7 +18363,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18477,7 +18477,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18591,7 +18591,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18705,7 +18705,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -18933,7 +18933,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19047,7 +19047,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19161,7 +19161,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19275,7 +19275,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19503,7 +19503,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19617,7 +19617,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19845,7 +19845,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19959,7 +19959,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20073,7 +20073,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20415,7 +20415,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20757,7 +20757,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -20985,7 +20985,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21099,7 +21099,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21213,7 +21213,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21555,7 +21555,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21783,7 +21783,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22125,7 +22125,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22239,7 +22239,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22695,7 +22695,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23037,7 +23037,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23151,7 +23151,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27369,7 +27369,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27483,7 +27483,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27597,7 +27597,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27711,7 +27711,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27825,7 +27825,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28053,7 +28053,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28167,7 +28167,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28281,7 +28281,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28395,7 +28395,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28509,7 +28509,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28623,7 +28623,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28737,7 +28737,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28851,7 +28851,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -28965,7 +28965,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29079,7 +29079,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29193,7 +29193,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29307,7 +29307,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29421,7 +29421,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29535,7 +29535,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29649,7 +29649,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29763,7 +29763,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -29877,7 +29877,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -29991,7 +29991,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30105,7 +30105,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30219,7 +30219,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30333,7 +30333,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30447,7 +30447,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30561,7 +30561,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30675,7 +30675,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30789,7 +30789,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30903,7 +30903,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31017,7 +31017,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31245,7 +31245,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31359,7 +31359,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31473,7 +31473,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31587,7 +31587,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31701,7 +31701,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31815,7 +31815,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32043,7 +32043,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32271,7 +32271,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32385,7 +32385,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32499,7 +32499,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32613,7 +32613,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32727,7 +32727,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -32841,7 +32841,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -32955,7 +32955,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33183,7 +33183,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33297,7 +33297,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33411,7 +33411,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33525,7 +33525,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33639,7 +33639,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33753,7 +33753,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -33867,7 +33867,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34095,7 +34095,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34209,7 +34209,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34323,7 +34323,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34437,7 +34437,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34551,7 +34551,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34665,7 +34665,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34779,7 +34779,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -34893,7 +34893,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36603,7 +36603,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36717,7 +36717,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -36945,7 +36945,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">
@@ -37059,7 +37059,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:54 PM PT</t>
+          <t>2026-07-11 10:44:54 PM PT</t>
         </is>
       </c>
       <c r="C321" t="n">
@@ -37173,7 +37173,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C322" t="n">
@@ -37287,7 +37287,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C323" t="n">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C324" t="n">
@@ -37515,7 +37515,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C325" t="n">
@@ -37629,7 +37629,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -37743,7 +37743,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C327" t="n">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C328" t="n">
@@ -37971,7 +37971,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C329" t="n">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C330" t="n">
@@ -38199,7 +38199,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C331" t="n">
@@ -38313,7 +38313,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C332" t="n">
@@ -38427,7 +38427,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C333" t="n">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C334" t="n">
@@ -38655,7 +38655,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C335" t="n">
@@ -38769,7 +38769,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C336" t="n">
@@ -38883,7 +38883,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>2026-07-11 10:42:55 PM PT</t>
+          <t>2026-07-11 10:44:55 PM PT</t>
         </is>
       </c>
       <c r="C337" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-11 10:46:57 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_11.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:54 PM PT</t>
+          <t>2026-07-11 10:46:54 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:54 PM PT</t>
+          <t>2026-07-11 10:46:54 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-11 10:44:55 PM PT</t>
+          <t>2026-07-11 10:46:55 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2517,7 +251